<commit_message>
Refine download plan ordering and expand large-provider ID examples
</commit_message>
<xml_diff>
--- a/workspace/input/input_generation/download_plan.xlsx
+++ b/workspace/input/input_generation/download_plan.xlsx
@@ -13,9 +13,9 @@
   <definedNames>
     <definedName name="id_opts_ensembl">'_lists'!$B$1:$B$348</definedName>
     <definedName name="id_opts_ensemblplants">'_lists'!$C$1:$C$266</definedName>
-    <definedName name="id_opts_ncbi">'_lists'!$D$1:$D$2</definedName>
-    <definedName name="id_opts_refseq">'_lists'!$E$1:$E$1</definedName>
-    <definedName name="id_opts_genbank">'_lists'!$F$1:$F$1</definedName>
+    <definedName name="id_opts_ncbi">'_lists'!$D$1:$D$5</definedName>
+    <definedName name="id_opts_refseq">'_lists'!$E$1:$E$5</definedName>
+    <definedName name="id_opts_genbank">'_lists'!$F$1:$F$5</definedName>
     <definedName name="id_opts_coge">'_lists'!$G$1:$G$1</definedName>
     <definedName name="id_opts_cngb">'_lists'!$H$1:$H$1</definedName>
     <definedName name="id_opts_flybase">'_lists'!$I$1:$I$12</definedName>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,413 +507,6 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>local_genome_path</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>cngb</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Streptococcus_urinalis</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Streptococcus_urinalis</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/CNGB/species_wise_original/Streptococcus_urinalis/Streptococcus_urinalis.cds.fa</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/CNGB/species_wise_original/Streptococcus_urinalis/Streptococcus_urinalis.gene.gff3</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Streptococcus_urinalis.cds.fa</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Streptococcus_urinalis.gene.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>coge</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>24739</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Arabidopsis_thaliana</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/CoGe/species_wise_original/Arabidopsis_thaliana/Arabidopsis_thaliana.coge.gid24739.cds.fa</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/CoGe/species_wise_original/Arabidopsis_thaliana/Arabidopsis_thaliana.gid24739.gff3</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Arabidopsis_thaliana.coge.gid24739.cds.fa</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Arabidopsis_thaliana.gid24739.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>ensembl</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>homo_sapiens</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>homo_sapiens</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/Ensembl/original_files/homo_sapiens.GRCh38.cds.all.fa</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/Ensembl/original_files/homo_sapiens.GRCh38.112.gff3</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>homo_sapiens.GRCh38.cds.all.fa</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>homo_sapiens.GRCh38.112.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>ensemblplants</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ostreococcus_lucimarinus</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Ostreococcus_lucimarinus</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/20230216_EnsemblPlants/original_files/Ostreococcus_lucimarinus.ASM9206v1.cds.all.fa</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/20230216_EnsemblPlants/original_files/Ostreococcus_lucimarinus.ASM9206v1.56.gff3</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Ostreococcus_lucimarinus.ASM9206v1.cds.all.fa</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Ostreococcus_lucimarinus.ASM9206v1.56.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>flybase</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Drosophila_melanogaster</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Drosophila_melanogaster</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/FlyBase/species_wise_original/Drosophila_melanogaster/dmel_r6.61.cds.fa</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/FlyBase/species_wise_original/Drosophila_melanogaster/dmel_r6.61.gff3</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>dmel_r6.61.cds.fa</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>dmel_r6.61.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>genbank</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>GCA_000001405.29</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>GCA_000001405.29</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_GenBank/species_wise_original/GCA_000001405.29/GCA_000001405.29_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_GenBank/species_wise_original/GCA_000001405.29/GCA_000001405.29_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>GCA_000001405.29_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>GCA_000001405.29_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>local</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Hydrocotyle_leucocephala_HAP1v2.1</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hydrocotyle_leucocephala_HAP1v2.1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/Local/species_wise_original/Hydrocotyle_leucocephala_HAP1v2.1/HleucocephalaHAP1_768_v2.1.cds_primaryTranscriptOnly.fa</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/Local/species_wise_original/Hydrocotyle_leucocephala_HAP1v2.1/HleucocephalaHAP1_768_v2.1.gene.gff3</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>HleucocephalaHAP1_768_v2.1.cds_primaryTranscriptOnly.fa</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>HleucocephalaHAP1_768_v2.1.gene.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ncbi</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_Genome/species_wise_original/GCF_000001405.40/GCF_000001405.40_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_Genome/species_wise_original/GCF_000001405.40/GCF_000001405.40_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>refseq</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_RefSeq/species_wise_original/GCF_000001405.40/GCF_000001405.40_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/NCBI_RefSeq/species_wise_original/GCF_000001405.40/GCF_000001405.40_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40_GRCh38.p14_cds_from_genomic.fna</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>GCF_000001405.40_GRCh38.p14_genomic.gff</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>vectorbase</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Anopheles_gambiae</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Anopheles_gambiae</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/VectorBase/species_wise_original/Anopheles_gambiae/anopheles_gambiae_pest.cds.fa</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/VectorBase/species_wise_original/Anopheles_gambiae/anopheles_gambiae_pest.gff3</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>anopheles_gambiae_pest.cds.fa</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>anopheles_gambiae_pest.gff3</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>wormbase</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Caenorhabditis_elegans</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Caenorhabditis_elegans</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/WormBase/species_wise_original/Caenorhabditis_elegans/celegans_prjna13758_ws290.cds.fa</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>file:///private/var/folders/xc/pydw8plj6vvf7mddh20v09sw0000gn/T/gg_seed_drm61ith/WormBase/species_wise_original/Caenorhabditis_elegans/celegans_prjna13758_ws290.gff3</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>celegans_prjna13758_ws290.cds.fa</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>celegans_prjna13758_ws290.gff3</t>
         </is>
       </c>
     </row>
@@ -922,7 +515,7 @@
     <dataValidation sqref="A2:A5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=_lists!$A$1:$A$11</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="ID candidates" error="This drop-down changes by provider. For large providers, model-organism IDs are shown as examples. You can still type any other ID value." type="list" errorStyle="information">
+    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="ID candidates" error="This drop-down changes by provider. For large providers, five model-organism IDs are shown as examples. You can still type any other ID value." type="list" errorStyle="information">
       <formula1>=INDIRECT("id_opts_"&amp;$A2)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1019,7 +612,17 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GCA_000001405.29 (Homo sapiens)</t>
+          <t>GCF_000001635.27 (Mus musculus)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>GCF_000001635.27 (Mus musculus)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GCA_000001635.9 (Mus musculus)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1054,6 +657,21 @@
           <t>aegilops_umbellulata (Aegilops umbellulata)</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>GCF_049306965.1 (Danio rerio)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>GCF_049306965.1 (Danio rerio)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GCA_049306965.1 (Danio rerio)</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>dgri_r1.05 (Drosophila grimshawi)</t>
@@ -1086,6 +704,21 @@
           <t>amborella_trichopoda (Amborella trichopoda)</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>GCF_000001215.4 (Drosophila melanogaster)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>GCF_000001215.4 (Drosophila melanogaster)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GCA_000001215.4 (Drosophila melanogaster)</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>dmel_r6.66 (Drosophila melanogaster)</t>
@@ -1116,6 +749,21 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>ananas_comosus (Ananas comosus)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>GCF_000002985.6 (Caenorhabditis elegans)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>GCF_000002985.6 (Caenorhabditis elegans)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GCA_000002985.3 (Caenorhabditis elegans)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">

</xml_diff>

<commit_message>
Unify NCBI providers and expand example ID options
</commit_message>
<xml_diff>
--- a/workspace/input/input_generation/download_plan.xlsx
+++ b/workspace/input/input_generation/download_plan.xlsx
@@ -14,14 +14,12 @@
     <definedName name="id_opts_ensembl">'_lists'!$B$1:$B$348</definedName>
     <definedName name="id_opts_ensemblplants">'_lists'!$C$1:$C$266</definedName>
     <definedName name="id_opts_ncbi">'_lists'!$D$1:$D$5</definedName>
-    <definedName name="id_opts_refseq">'_lists'!$E$1:$E$5</definedName>
-    <definedName name="id_opts_genbank">'_lists'!$F$1:$F$5</definedName>
-    <definedName name="id_opts_coge">'_lists'!$G$1:$G$1</definedName>
-    <definedName name="id_opts_cngb">'_lists'!$H$1:$H$1</definedName>
-    <definedName name="id_opts_flybase">'_lists'!$I$1:$I$12</definedName>
-    <definedName name="id_opts_wormbase">'_lists'!$J$1:$J$248</definedName>
-    <definedName name="id_opts_vectorbase">'_lists'!$K$1:$K$131</definedName>
-    <definedName name="id_opts_local">'_lists'!$L$1:$L$1</definedName>
+    <definedName name="id_opts_coge">'_lists'!$E$1:$E$5</definedName>
+    <definedName name="id_opts_cngb">'_lists'!$F$1:$F$1</definedName>
+    <definedName name="id_opts_flybase">'_lists'!$G$1:$G$12</definedName>
+    <definedName name="id_opts_wormbase">'_lists'!$H$1:$H$248</definedName>
+    <definedName name="id_opts_vectorbase">'_lists'!$I$1:$I$131</definedName>
+    <definedName name="id_opts_local">'_lists'!$J$1:$J$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -513,9 +511,9 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="A2:A5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=_lists!$A$1:$A$11</formula1>
+      <formula1>=_lists!$A$1:$A$9</formula1>
     </dataValidation>
-    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="ID candidates" error="This drop-down changes by provider. For large providers, five model-organism IDs are shown as examples. You can still type any other ID value." type="list" errorStyle="information">
+    <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="ID candidates" error="This drop-down changes by provider. For provider=ncbi, five model-organism IDs are shown as examples. You can still type any other ID value." type="list" errorStyle="information">
       <formula1>=INDIRECT("id_opts_"&amp;$A2)</formula1>
     </dataValidation>
   </dataValidations>
@@ -529,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L348"/>
+  <dimension ref="A1:J348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,40 +553,30 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>GCF_000001405.40 (Homo sapiens)</t>
+          <t>24739 (Arabidopsis thaliana)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>GCA_000001405.29 (Homo sapiens)</t>
+          <t>CNA0012345 (Homo sapiens)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>24739 (Arabidopsis thaliana)</t>
+          <t>dana_r1.06 (Drosophila ananassae)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>CNA0012345 (Homo sapiens)</t>
+          <t>acanthocheilonema_viteae_prjeb1697 (acanthocheilonema viteae)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>dana_r1.06 (Drosophila ananassae)</t>
+          <t>Aaegypti (A. aegypti)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
-        <is>
-          <t>acanthocheilonema_viteae_prjeb1697 (acanthocheilonema viteae)</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>Aaegypti (A. aegypti)</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
         <is>
           <t>/absolute/path/to/local/species_dir</t>
         </is>
@@ -612,30 +600,25 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GCF_000001635.27 (Mus musculus)</t>
+          <t>GCA_000001635.9 (Mus musculus)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GCF_000001635.27 (Mus musculus)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>GCA_000001635.9 (Mus musculus)</t>
+          <t>29177 (Oryza sativa)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>dere_r1.05 (Drosophila erecta)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>acrobeloides_nanus_prjeb26554 (acrobeloides nanus)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
-        <is>
-          <t>dere_r1.05 (Drosophila erecta)</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>acrobeloides_nanus_prjeb26554 (acrobeloides nanus)</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
         <is>
           <t>AaegyptiAag2 (A. aegypti)</t>
         </is>
@@ -664,25 +647,20 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>GCF_049306965.1 (Danio rerio)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>GCA_049306965.1 (Danio rerio)</t>
+          <t>42091 (Zea mays)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>dgri_r1.05 (Drosophila grimshawi)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>allodiplogaster_sudhausi_prjeb48369 (allodiplogaster sudhausi)</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>dgri_r1.05 (Drosophila grimshawi)</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>allodiplogaster_sudhausi_prjeb48369 (allodiplogaster sudhausi)</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
         <is>
           <t>AaegyptiLVP_AGWG (A. aegypti)</t>
         </is>
@@ -691,7 +669,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>refseq</t>
+          <t>coge</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -706,30 +684,25 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GCF_000001215.4 (Drosophila melanogaster)</t>
+          <t>GCA_000001215.4 (Drosophila melanogaster)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>GCF_000001215.4 (Drosophila melanogaster)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>GCA_000001215.4 (Drosophila melanogaster)</t>
+          <t>78085 (Drosophila melanogaster)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>dmel_r6.66 (Drosophila melanogaster)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>ancylostoma_caninum_prjna72585 (ancylostoma caninum)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
-        <is>
-          <t>dmel_r6.66 (Drosophila melanogaster)</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>ancylostoma_caninum_prjna72585 (ancylostoma caninum)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
         <is>
           <t>Aalbimanus (A. albimanus)</t>
         </is>
@@ -738,7 +711,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>genbank</t>
+          <t>cngb</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -758,25 +731,20 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>GCF_000002985.6 (Caenorhabditis elegans)</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>GCA_000002985.3 (Caenorhabditis elegans)</t>
+          <t>72417 (Caenorhabditis elegans)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>dmoj_r1.04 (Drosophila mojavensis)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>ancylostoma_ceylanicum_prjna231479 (ancylostoma ceylanicum)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
-        <is>
-          <t>dmoj_r1.04 (Drosophila mojavensis)</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ancylostoma_ceylanicum_prjna231479 (ancylostoma ceylanicum)</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
         <is>
           <t>AalbimanusSTECLA (A. albimanus)</t>
         </is>
@@ -785,7 +753,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>coge</t>
+          <t>flybase</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -798,17 +766,17 @@
           <t>arabidopsis_halleri (Arabidopsis halleri)</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>dper_r1.3 (Drosophila persimilis)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>ancylostoma_ceylanicum_prjna72583 (ancylostoma ceylanicum)</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
-        <is>
-          <t>dper_r1.3 (Drosophila persimilis)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>ancylostoma_ceylanicum_prjna72583 (ancylostoma ceylanicum)</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
         <is>
           <t>AalbimanusSTECLA2020 (A. albimanus)</t>
         </is>
@@ -817,7 +785,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cngb</t>
+          <t>wormbase</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -830,17 +798,17 @@
           <t>arabidopsis_lyrata (Arabidopsis lyrata)</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>dpse_r3.04 (Drosophila pseudoobscura)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>ancylostoma_duodenale_prjna72581 (ancylostoma duodenale)</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
-        <is>
-          <t>dpse_r3.04 (Drosophila pseudoobscura)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>ancylostoma_duodenale_prjna72581 (ancylostoma duodenale)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
         <is>
           <t>Aalbopictus (A. albopictus)</t>
         </is>
@@ -849,7 +817,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>flybase</t>
+          <t>vectorbase</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -862,17 +830,17 @@
           <t>arabidopsis_thaliana (Arabidopsis thaliana)</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>dsec_r1.3 (Drosophila sechellia)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>angiostrongylus_cantonensis_prjeb493 (angiostrongylus cantonensis)</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
-        <is>
-          <t>dsec_r1.3 (Drosophila sechellia)</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>angiostrongylus_cantonensis_prjeb493 (angiostrongylus cantonensis)</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
         <is>
           <t>AalbopictusC6-36 (A. albopictus)</t>
         </is>
@@ -881,7 +849,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>wormbase</t>
+          <t>local</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -894,28 +862,23 @@
           <t>arabis_alpina (Arabis alpina)</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>dsim_r2.02 (Drosophila simulans)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>angiostrongylus_cantonensis_prjna350391 (angiostrongylus cantonensis)</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>dsim_r2.02 (Drosophila simulans)</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>angiostrongylus_cantonensis_prjna350391 (angiostrongylus cantonensis)</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
           <t>AalbopictusFoshan (A. albopictus)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>vectorbase</t>
-        </is>
-      </c>
       <c r="B10" t="inlineStr">
         <is>
           <t>anas_platyrhynchos_platyrhynchos (Duck)</t>
@@ -926,28 +889,23 @@
           <t>arachis_hypogaea (Arachis hypogaea)</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>dvir_r1.07 (Drosophila virilis)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>angiostrongylus_costaricensis_prjeb494 (angiostrongylus costaricensis)</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>dvir_r1.07 (Drosophila virilis)</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>angiostrongylus_costaricensis_prjeb494 (angiostrongylus costaricensis)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
           <t>AalbopictusFoshanFPA (A. albopictus)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>local</t>
-        </is>
-      </c>
       <c r="B11" t="inlineStr">
         <is>
           <t>anas_zonorhyncha (Eastern spot-billed duck)</t>
@@ -958,17 +916,17 @@
           <t>asparagus_officinalis (Asparagus officinalis)</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>dwil_r1.05 (Drosophila willistoni)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>angiostrongylus_vasorum_prjna663250 (angiostrongylus vasorum)</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
-        <is>
-          <t>dwil_r1.05 (Drosophila willistoni)</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>angiostrongylus_vasorum_prjna663250 (angiostrongylus vasorum)</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
         <is>
           <t>Aaquasalis (A. aquasalis)</t>
         </is>
@@ -985,17 +943,17 @@
           <t>avena_atlantica_gca910589765v1cm (Avena atlantica gca910589765v1cm)</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>dyak_r1.05 (Drosophila yakuba)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>anisakis_simplex_prjeb496 (anisakis simplex)</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
-        <is>
-          <t>dyak_r1.05 (Drosophila yakuba)</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>anisakis_simplex_prjeb496 (anisakis simplex)</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
         <is>
           <t>AaquasalisAaquGF1 (A. aquasalis)</t>
         </is>
@@ -1012,12 +970,12 @@
           <t>avena_byzantina_gca910574625v1cm (Avena byzantina gca910574625v1cm)</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>aphelenchoides_bicaudatus_prjna834627 (aphelenchoides bicaudatus)</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>AarabiensisDongola (A. arabiensis)</t>
         </is>
@@ -1034,12 +992,12 @@
           <t>avena_eriantha_gca910589775v1cm (Avena eriantha gca910589775v1cm)</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>aphelenchoides_fujianensis_prjna834627 (aphelenchoides fujianensis)</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>AarabiensisDONGOLA2021 (A. arabiensis)</t>
         </is>
@@ -1056,12 +1014,12 @@
           <t>avena_insularis_gca910574615v1cm (Avena insularis gca910574615v1cm)</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>ascaris_lumbricoides_prjeb4950 (ascaris lumbricoides)</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>Aatroparvus (A. atroparvus)</t>
         </is>
@@ -1078,12 +1036,12 @@
           <t>avena_longiglumis_gca910589755v1cm (Avena longiglumis gca910589755v1cm)</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>ascaris_suum_prjna62057 (ascaris suum)</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>AatroparvusEBRO (A. atroparvus)</t>
         </is>
@@ -1100,12 +1058,12 @@
           <t>avena_occidentalis_gca947310975v1cm (Avena occidentalis gca947310975v1cm)</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>ascaris_suum_prjna80881 (ascaris suum)</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="I17" t="inlineStr">
         <is>
           <t>AbellatorAbelBR1 (A. bellator)</t>
         </is>
@@ -1122,12 +1080,12 @@
           <t>avena_sativa_gca947310255v1cm (Avena sativa gca947310255v1cm)</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>atriophallophorus_winterbourni_prjna636673 (atriophallophorus winterbourni)</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="I18" t="inlineStr">
         <is>
           <t>Achristyi (A. christyi)</t>
         </is>
@@ -1144,12 +1102,12 @@
           <t>avena_sativa_gca947310285v1cm (Avena sativa gca947310285v1cm)</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>auanema_ju1783_prjeb51845 (auanema ju1783)</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="I19" t="inlineStr">
         <is>
           <t>AchristyiACHKN1017 (A. christyi)</t>
         </is>
@@ -1166,12 +1124,12 @@
           <t>avena_sativa_gca947310875v1cm (Avena sativa gca947310875v1cm)</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>bradynema_listronoti_prjna842945 (bradynema listronoti)</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>AcoluzziiAcolN3 (A. coluzzii)</t>
         </is>
@@ -1188,12 +1146,12 @@
           <t>avena_sativa_gca947311085v1cm (Avena sativa gca947311085v1cm)</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>brugia_malayi_prjna10729 (brugia malayi)</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>AcoluzziiMali-NIH (A. coluzzii)</t>
         </is>
@@ -1210,12 +1168,12 @@
           <t>avena_sativa_gca947311135v1cm (Avena sativa gca947311135v1cm)</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>brugia_pahangi_prjeb497 (brugia pahangi)</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>AcoluzziiMOPTI (A. coluzzii)</t>
         </is>
@@ -1232,12 +1190,12 @@
           <t>avena_sativa_gca947311155v1cm (Avena sativa gca947311155v1cm)</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>brugia_timori_prjeb4663 (brugia timori)</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
+      <c r="I23" t="inlineStr">
         <is>
           <t>AcoluzziiNgousso (A. coluzzii)</t>
         </is>
@@ -1254,12 +1212,12 @@
           <t>avena_sativa_gca947311165v1cm (Avena sativa gca947311165v1cm)</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>bunonema_rgd898_prjna655932 (bunonema rgd898)</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="I24" t="inlineStr">
         <is>
           <t>AcoustaniAcouGA1 (A. coustani)</t>
         </is>
@@ -1276,12 +1234,12 @@
           <t>avena_sativa_gca947311225v1cm (Avena sativa gca947311225v1cm)</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>bursaphelenchus_okinawaensis_prjeb40023 (bursaphelenchus okinawaensis)</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
+      <c r="I25" t="inlineStr">
         <is>
           <t>AcruziiAcruBR1 (A. cruzii)</t>
         </is>
@@ -1298,12 +1256,12 @@
           <t>avena_sativa_gca947311235v1cm (Avena sativa gca947311235v1cm)</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>bursaphelenchus_xylophilus_prjea64437 (bursaphelenchus xylophilus)</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
+      <c r="I26" t="inlineStr">
         <is>
           <t>Aculicifacies (A. culicifacies)</t>
         </is>
@@ -1320,12 +1278,12 @@
           <t>avena_sativa_gca947311295v1cm (Avena sativa gca947311295v1cm)</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>bursaphelenchus_xylophilus_prjeb40022 (bursaphelenchus xylophilus)</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
+      <c r="I27" t="inlineStr">
         <is>
           <t>AculicifaciesA-37 (A. culicifacies)</t>
         </is>
@@ -1342,12 +1300,12 @@
           <t>avena_sativa_gca947311345v1cm (Avena sativa gca947311345v1cm)</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>caenorhabditis_angaria_prjna51225 (caenorhabditis angaria)</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
+      <c r="I28" t="inlineStr">
         <is>
           <t>AdarlingiAdarGF1 (A. darlingi)</t>
         </is>
@@ -1364,12 +1322,12 @@
           <t>avena_sativa_gca947311355v1cm (Avena sativa gca947311355v1cm)</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>caenorhabditis_auriculariae_prjeb40642 (caenorhabditis auriculariae)</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>AdarlingiCoari (A. darlingi)</t>
         </is>
@@ -1386,12 +1344,12 @@
           <t>avena_sativa_gca947311365v1cm (Avena sativa gca947311365v1cm)</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>caenorhabditis_becei_prjeb28243 (caenorhabditis becei)</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
+      <c r="I30" t="inlineStr">
         <is>
           <t>Adirus (A. dirus)</t>
         </is>
@@ -1408,12 +1366,12 @@
           <t>avena_sativa_gca947311525v1cm (Avena sativa gca947311525v1cm)</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>caenorhabditis_bovis_prjeb34497 (caenorhabditis bovis)</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
+      <c r="I31" t="inlineStr">
         <is>
           <t>AdirusWRAIR2 (A. dirus)</t>
         </is>
@@ -1430,12 +1388,12 @@
           <t>avena_sativa_gca947311555v1cm (Avena sativa gca947311555v1cm)</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>caenorhabditis_brenneri_prjna20035 (caenorhabditis brenneri)</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
+      <c r="I32" t="inlineStr">
         <is>
           <t>Aepiroticus (A. epiroticus)</t>
         </is>
@@ -1452,12 +1410,12 @@
           <t>avena_sativa_gca947311775v1cm (Avena sativa gca947311775v1cm)</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>caenorhabditis_briggsae_prjna10731 (caenorhabditis briggsae)</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
+      <c r="I33" t="inlineStr">
         <is>
           <t>AepiroticusEpiroticus2 (A. epiroticus)</t>
         </is>
@@ -1474,12 +1432,12 @@
           <t>avena_sativa_gca947311915v1cm (Avena sativa gca947311915v1cm)</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>caenorhabditis_elegans_prjna13758 (caenorhabditis elegans)</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>Afarauti (A. farauti)</t>
         </is>
@@ -1496,12 +1454,12 @@
           <t>avena_sativa_gca947311925v1cm (Avena sativa gca947311925v1cm)</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>caenorhabditis_inopinata_prjdb5687 (caenorhabditis inopinata)</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
+      <c r="I35" t="inlineStr">
         <is>
           <t>AfarautiFAR1 (A. farauti)</t>
         </is>
@@ -1518,12 +1476,12 @@
           <t>avena_sativa_gca947312425v1cm (Avena sativa gca947312425v1cm)</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>caenorhabditis_japonica_prjna12591 (caenorhabditis japonica)</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
+      <c r="I36" t="inlineStr">
         <is>
           <t>Afunestus (A. funestus)</t>
         </is>
@@ -1540,12 +1498,12 @@
           <t>avena_sativa_gca951802345v1cm (Avena sativa gca951802345v1cm)</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>caenorhabditis_latens_prjna248912 (caenorhabditis latens)</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>AfunestusAfunGA1 (A. funestus)</t>
         </is>
@@ -1562,12 +1520,12 @@
           <t>avena_sativa_gca951802355v1cm (Avena sativa gca951802355v1cm)</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>caenorhabditis_nigoni_prjna384657 (caenorhabditis nigoni)</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
+      <c r="I38" t="inlineStr">
         <is>
           <t>AfunestusFUMOZ (A. funestus)</t>
         </is>
@@ -1584,12 +1542,12 @@
           <t>avena_sativa_gca951802365v1cm (Avena sativa gca951802365v1cm)</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>caenorhabditis_panamensis_prjeb28259 (caenorhabditis panamensis)</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Agambiae (A. gambiae)</t>
         </is>
@@ -1606,12 +1564,12 @@
           <t>avena_sativa_ot3098 (Avena sativa ot3098)</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>caenorhabditis_parvicauda_prjeb12595 (caenorhabditis parvicauda)</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>AgambiaeIfakara (A. gambiae)</t>
         </is>
@@ -1628,12 +1586,12 @@
           <t>avena_sativa_sang (Avena sativa sang)</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>caenorhabditis_quiockensis_prjeb11354 (caenorhabditis quiockensis)</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>AgambiaePEST (A. gambiae)</t>
         </is>
@@ -1650,12 +1608,12 @@
           <t>avena_sterilis_gca947313225v1cm (Avena sterilis gca947313225v1cm)</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>caenorhabditis_remanei_prjna248909 (caenorhabditis remanei)</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="I42" t="inlineStr">
         <is>
           <t>AgambiaePimperena (A. gambiae)</t>
         </is>
@@ -1672,12 +1630,12 @@
           <t>avena_sterilis_gca947313515v1cm (Avena sterilis gca947313515v1cm)</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>caenorhabditis_remanei_prjna248911 (caenorhabditis remanei)</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>AmaculatumSK-2019 (A. maculatum)</t>
         </is>
@@ -1694,12 +1652,12 @@
           <t>beta_vulgaris (Beta vulgaris)</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>caenorhabditis_remanei_prjna53967 (caenorhabditis remanei)</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="I44" t="inlineStr">
         <is>
           <t>Amaculatus (A. maculatus)</t>
         </is>
@@ -1716,12 +1674,12 @@
           <t>brachypodium_distachyon (Brachypodium distachyon)</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>caenorhabditis_remanei_prjna577507 (caenorhabditis remanei)</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="I45" t="inlineStr">
         <is>
           <t>Amaculatusmaculatus3 (A. maculatusmaculatus)</t>
         </is>
@@ -1738,12 +1696,12 @@
           <t>brassica_juncea (Brassica juncea)</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>caenorhabditis_sinica_prjna194557 (caenorhabditis sinica)</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>AmaculipalpisAmacGA1 (A. maculipalpis)</t>
         </is>
@@ -1760,12 +1718,12 @@
           <t>brassica_napus (Brassica napus)</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>caenorhabditis_sulstoni_prjeb12601 (caenorhabditis sulstoni)</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="I47" t="inlineStr">
         <is>
           <t>AmarshalliiAmarGA1 (A. marshallii)</t>
         </is>
@@ -1782,12 +1740,12 @@
           <t>brassica_oleracea (Brassica oleracea)</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>caenorhabditis_tribulationis_prjeb12608 (caenorhabditis tribulationis)</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
+      <c r="I48" t="inlineStr">
         <is>
           <t>Amelas (A. melas)</t>
         </is>
@@ -1804,12 +1762,12 @@
           <t>brassica_rapa (Brassica rapa)</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>caenorhabditis_tropicalis_prjna53597 (caenorhabditis tropicalis)</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>AmelasCM1001059_A (A. melas)</t>
         </is>
@@ -1826,12 +1784,12 @@
           <t>brassica_rapa_ro18 (Brassica rapa ro18)</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>caenorhabditis_uteleia_prjeb12600 (caenorhabditis uteleia)</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>AmerusMAF (A. merus)</t>
         </is>
@@ -1848,12 +1806,12 @@
           <t>brassica_rapa_z1 (Brassica rapa z1)</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>caenorhabditis_waitukubuli_prjeb12602 (caenorhabditis waitukubuli)</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
+      <c r="I51" t="inlineStr">
         <is>
           <t>AmerusMAF2021 (A. merus)</t>
         </is>
@@ -1870,12 +1828,12 @@
           <t>cajanus_cajan (Cajanus cajan)</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>caenorhabditis_zanzibari_prjeb12596 (caenorhabditis zanzibari)</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>Aminimus (A. minimus)</t>
         </is>
@@ -1892,12 +1850,12 @@
           <t>camelina_sativa (Camelina sativa)</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>cercopithifilaria_johnstoni_prjeb47283 (cercopithifilaria johnstoni)</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="I53" t="inlineStr">
         <is>
           <t>AminimusMINIMUS1 (A. minimus)</t>
         </is>
@@ -1914,12 +1872,12 @@
           <t>cannabis_sativa_female (Cannabis sativa female)</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>clonorchis_sinensis_prjda72781 (clonorchis sinensis)</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
+      <c r="I54" t="inlineStr">
         <is>
           <t>AmouchetiAmouCM1 (A. moucheti)</t>
         </is>
@@ -1936,12 +1894,12 @@
           <t>capsicum_annuum (Capsicum annuum)</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>clonorchis_sinensis_prjna386618 (clonorchis sinensis)</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
+      <c r="I55" t="inlineStr">
         <is>
           <t>AniliAnilCM1 (A. nili)</t>
         </is>
@@ -1958,12 +1916,12 @@
           <t>chara_braunii (Chara braunii)</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>cylicocyclus_nassatus_prjeb63274 (cylicocyclus nassatus)</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="I56" t="inlineStr">
         <is>
           <t>Aquadriannulatus (A. quadriannulatus)</t>
         </is>
@@ -1980,12 +1938,12 @@
           <t>chenopodium_quinoa (Chenopodium quinoa)</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>cylicostephanus_goldi_prjeb498 (cylicostephanus goldi)</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>AquadriannulatusSANGWE (A. quadriannulatus)</t>
         </is>
@@ -2002,12 +1960,12 @@
           <t>chlamydomonas_reinhardtii (Chlamydomonas reinhardtii)</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>dibothriocephalus_latus_prjeb1206 (dibothriocephalus latus)</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>AsinensisChina (A. sinensis)</t>
         </is>
@@ -2024,12 +1982,12 @@
           <t>chondrus_crispus (Chondrus crispus)</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>dicrocoelium_dendriticum_prjeb44434 (dicrocoelium dendriticum)</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>AsinensisSINENSIS (A. sinensis)</t>
         </is>
@@ -2046,12 +2004,12 @@
           <t>citrullus_lanatus (Citrullus lanatus)</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="H60" t="inlineStr">
         <is>
           <t>dictyocaulus_viviparus_prjeb5116 (dictyocaulus viviparus)</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
+      <c r="I60" t="inlineStr">
         <is>
           <t>Astephensi (A. stephensi)</t>
         </is>
@@ -2068,12 +2026,12 @@
           <t>citrus_clementina (Citrus clementina)</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="H61" t="inlineStr">
         <is>
           <t>dictyocaulus_viviparus_prjna72587 (dictyocaulus viviparus)</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>AstephensiIndian (A. stephensi)</t>
         </is>
@@ -2090,12 +2048,12 @@
           <t>coffea_canephora (Coffea canephora)</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="H62" t="inlineStr">
         <is>
           <t>diplogasteroides_magnus_prjna655932 (diplogasteroides magnus)</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
+      <c r="I62" t="inlineStr">
         <is>
           <t>AstephensiSDA-500 (A. stephensi)</t>
         </is>
@@ -2112,12 +2070,12 @@
           <t>corchorus_capsularis (Corchorus capsularis)</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
+      <c r="H63" t="inlineStr">
         <is>
           <t>diploscapter_coronatus_prjdb3143 (diploscapter coronatus)</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
+      <c r="I63" t="inlineStr">
         <is>
           <t>AstephensiUCISS2018 (A. stephensi)</t>
         </is>
@@ -2134,12 +2092,12 @@
           <t>corylus_avellana (Corylus avellana)</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr">
+      <c r="H64" t="inlineStr">
         <is>
           <t>diploscapter_pachys_prjna280107 (diploscapter pachys)</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
+      <c r="I64" t="inlineStr">
         <is>
           <t>AziemanniAzieGA1 (A. ziemanni)</t>
         </is>
@@ -2156,12 +2114,12 @@
           <t>corymbia_citriodora (Corymbia citriodora)</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr">
+      <c r="H65" t="inlineStr">
         <is>
           <t>dirofilaria_immitis_prjeb1797 (dirofilaria immitis)</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
+      <c r="I65" t="inlineStr">
         <is>
           <t>Bglabrata (B. glabrata)</t>
         </is>
@@ -2178,12 +2136,12 @@
           <t>cucumis_melo (Cucumis melo)</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr">
+      <c r="H66" t="inlineStr">
         <is>
           <t>dirofilaria_immitis_prjna723804 (dirofilaria immitis)</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
+      <c r="I66" t="inlineStr">
         <is>
           <t>BglabrataBB02 (B. glabrata)</t>
         </is>
@@ -2200,12 +2158,12 @@
           <t>cucumis_sativus (Cucumis sativus)</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr">
+      <c r="H67" t="inlineStr">
         <is>
           <t>ditylenchus_destructor_prjna312427 (ditylenchus destructor)</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
+      <c r="I67" t="inlineStr">
         <is>
           <t>BglabrataXG47 (B. glabrata)</t>
         </is>
@@ -2222,12 +2180,12 @@
           <t>cyanidioschyzon_merolae (Cyanidioschyzon merolae)</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr">
+      <c r="H68" t="inlineStr">
         <is>
           <t>ditylenchus_destructor_prjna800207 (ditylenchus destructor)</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
+      <c r="I68" t="inlineStr">
         <is>
           <t>Build_number (B. uild)</t>
         </is>
@@ -2244,12 +2202,12 @@
           <t>cynara_cardunculus (Cynara cardunculus)</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr">
+      <c r="H69" t="inlineStr">
         <is>
           <t>ditylenchus_dipsaci_prjna498219 (ditylenchus dipsaci)</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
+      <c r="I69" t="inlineStr">
         <is>
           <t>Clectularius (C. lectularius)</t>
         </is>
@@ -2266,12 +2224,12 @@
           <t>daucus_carota (Daucus carota)</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr">
+      <c r="H70" t="inlineStr">
         <is>
           <t>dracunculus_medinensis_prjeb500 (dracunculus medinensis)</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
+      <c r="I70" t="inlineStr">
         <is>
           <t>ClectulariusHarlan (C. lectularius)</t>
         </is>
@@ -2288,12 +2246,12 @@
           <t>digitaria_exilis (Digitaria exilis)</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>echinococcus_canadensis_prjeb8992 (echinococcus canadensis)</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
+      <c r="I71" t="inlineStr">
         <is>
           <t>Cquinquefasciatus (C. quinquefasciatus)</t>
         </is>
@@ -2310,12 +2268,12 @@
           <t>dioscorea_rotundata (Dioscorea rotundata)</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr">
+      <c r="H72" t="inlineStr">
         <is>
           <t>echinococcus_granulosus_prjeb121 (echinococcus granulosus)</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
+      <c r="I72" t="inlineStr">
         <is>
           <t>CquinquefasciatusJHB2020 (C. quinquefasciatus)</t>
         </is>
@@ -2332,12 +2290,12 @@
           <t>echinochloa_crusgalli (Echinochloa crusgalli)</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr">
+      <c r="H73" t="inlineStr">
         <is>
           <t>echinococcus_granulosus_prjna182977 (echinococcus granulosus)</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
+      <c r="I73" t="inlineStr">
         <is>
           <t>CquinquefasciatusJohannesburg (C. quinquefasciatus)</t>
         </is>
@@ -2354,12 +2312,12 @@
           <t>eragrostis_curvula (Eragrostis curvula)</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="H74" t="inlineStr">
         <is>
           <t>echinococcus_granulosus_prjna754835 (echinococcus granulosus)</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>Csonorensis (C. sonorensis)</t>
         </is>
@@ -2376,12 +2334,12 @@
           <t>eragrostis_tef (Eragrostis tef)</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr">
+      <c r="H75" t="inlineStr">
         <is>
           <t>echinococcus_multilocularis_prjeb122 (echinococcus multilocularis)</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
+      <c r="I75" t="inlineStr">
         <is>
           <t>CsonorensisPIR-s-3 (C. sonorensis)</t>
         </is>
@@ -2398,12 +2356,12 @@
           <t>eucalyptus_grandis (Eucalyptus grandis)</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr">
+      <c r="H76" t="inlineStr">
         <is>
           <t>echinococcus_oligarthrus_prjeb31222 (echinococcus oligarthrus)</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
+      <c r="I76" t="inlineStr">
         <is>
           <t>Dandersoni (D. andersoni)</t>
         </is>
@@ -2420,12 +2378,12 @@
           <t>eutrema_salsugineum (Eutrema salsugineum)</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr">
+      <c r="H77" t="inlineStr">
         <is>
           <t>echinostoma_caproni_prjeb1207 (echinostoma caproni)</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
+      <c r="I77" t="inlineStr">
         <is>
           <t>DandersoniqqDerAnde1.1 (D. andersoniqq)</t>
         </is>
@@ -2442,12 +2400,12 @@
           <t>ficus_carica (Ficus carica)</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr">
+      <c r="H78" t="inlineStr">
         <is>
           <t>elaeophora_elaphi_prjeb502 (elaeophora elaphi)</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
+      <c r="I78" t="inlineStr">
         <is>
           <t>DandersoniqqDerAnde1.2 (D. andersoniqq)</t>
         </is>
@@ -2464,12 +2422,12 @@
           <t>fraxinus_excelsior (Fraxinus excelsior)</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr">
+      <c r="H79" t="inlineStr">
         <is>
           <t>enoplolaimus_lenunculus_prjna953805 (enoplolaimus lenunculus)</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
+      <c r="I79" t="inlineStr">
         <is>
           <t>Dmelanogaster (D. melanogaster)</t>
         </is>
@@ -2486,12 +2444,12 @@
           <t>galdieria_sulphuraria (Galdieria sulphuraria)</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr">
+      <c r="H80" t="inlineStr">
         <is>
           <t>enterobius_vermicularis_prjeb503 (enterobius vermicularis)</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
+      <c r="I80" t="inlineStr">
         <is>
           <t>Dmelanogasteriso-1 (D. melanogasteriso)</t>
         </is>
@@ -2508,12 +2466,12 @@
           <t>glycine_max (Glycine max)</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr">
+      <c r="H81" t="inlineStr">
         <is>
           <t>epsilonema_zab32_prjna953805 (epsilonema zab32)</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="I81" t="inlineStr">
         <is>
           <t>DsilvarumDsil-2018 (D. silvarum)</t>
         </is>
@@ -2530,12 +2488,12 @@
           <t>glycine_soja (Glycine soja)</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr">
+      <c r="H82" t="inlineStr">
         <is>
           <t>fasciola_gigantica_prjna230515 (fasciola gigantica)</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr">
+      <c r="I82" t="inlineStr">
         <is>
           <t>Gausteni (G. austeni)</t>
         </is>
@@ -2552,12 +2510,12 @@
           <t>gossypium_raimondii (Gossypium raimondii)</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr">
+      <c r="H83" t="inlineStr">
         <is>
           <t>fasciola_hepatica_prjeb58756 (fasciola hepatica)</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr">
+      <c r="I83" t="inlineStr">
         <is>
           <t>GausteniTTRI (G. austeni)</t>
         </is>
@@ -2574,12 +2532,12 @@
           <t>helianthus_annuus (Helianthus annuus)</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr">
+      <c r="H84" t="inlineStr">
         <is>
           <t>fasciola_hepatica_prjna179522 (fasciola hepatica)</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
+      <c r="I84" t="inlineStr">
         <is>
           <t>Gbrevipalpis (G. brevipalpis)</t>
         </is>
@@ -2596,12 +2554,12 @@
           <t>hordeum_vulgare (Hordeum vulgare)</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr">
+      <c r="H85" t="inlineStr">
         <is>
           <t>fasciolopsis_buski_prjna284521 (fasciolopsis buski)</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
+      <c r="I85" t="inlineStr">
         <is>
           <t>GbrevipalpisIAEA (G. brevipalpis)</t>
         </is>
@@ -2618,12 +2576,12 @@
           <t>hordeum_vulgare_10tj18 (Hordeum vulgare 10tj18)</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr">
+      <c r="H86" t="inlineStr">
         <is>
           <t>globodera_pallida_prjeb123 (globodera pallida)</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
+      <c r="I86" t="inlineStr">
         <is>
           <t>GfuscipesIAEA (G. fuscipes)</t>
         </is>
@@ -2640,12 +2598,12 @@
           <t>hordeum_vulgare_aizu6 (Hordeum vulgare aizu6)</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr">
+      <c r="H87" t="inlineStr">
         <is>
           <t>globodera_pallida_prjna702104 (globodera pallida)</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr">
+      <c r="I87" t="inlineStr">
         <is>
           <t>GfuscipesIAEA2018 (G. fuscipes)</t>
         </is>
@@ -2662,12 +2620,12 @@
           <t>hordeum_vulgare_akashinriki (Hordeum vulgare akashinriki)</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr">
+      <c r="H88" t="inlineStr">
         <is>
           <t>globodera_pallida_prjna764088 (globodera pallida)</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
+      <c r="I88" t="inlineStr">
         <is>
           <t>Gmorsitans (G. morsitans)</t>
         </is>
@@ -2684,12 +2642,12 @@
           <t>hordeum_vulgare_barke (Hordeum vulgare barke)</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr">
+      <c r="H89" t="inlineStr">
         <is>
           <t>globodera_rostochiensis_prjeb13504 (globodera rostochiensis)</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
+      <c r="I89" t="inlineStr">
         <is>
           <t>GmorsitansYale (G. morsitans)</t>
         </is>
@@ -2706,12 +2664,12 @@
           <t>hordeum_vulgare_bonus (Hordeum vulgare bonus)</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr">
+      <c r="H90" t="inlineStr">
         <is>
           <t>gongylonema_pulchrum_prjeb505 (gongylonema pulchrum)</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
+      <c r="I90" t="inlineStr">
         <is>
           <t>Gpallidipes (G. pallidipes)</t>
         </is>
@@ -2728,12 +2686,12 @@
           <t>hordeum_vulgare_bowman (Hordeum vulgare bowman)</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr">
+      <c r="H91" t="inlineStr">
         <is>
           <t>gyrodactylus_bullatarudis_prjna532341 (gyrodactylus bullatarudis)</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
+      <c r="I91" t="inlineStr">
         <is>
           <t>GpallidipesIAEA (G. pallidipes)</t>
         </is>
@@ -2750,12 +2708,12 @@
           <t>hordeum_vulgare_chikurinibaraki1 (Hordeum vulgare chikurinibaraki1)</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr">
+      <c r="H92" t="inlineStr">
         <is>
           <t>gyrodactylus_salaris_prjna244375 (gyrodactylus salaris)</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr">
+      <c r="I92" t="inlineStr">
         <is>
           <t>Gpalpalis (G. palpalis)</t>
         </is>
@@ -2772,12 +2730,12 @@
           <t>hordeum_vulgare_foma (Hordeum vulgare foma)</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr">
+      <c r="H93" t="inlineStr">
         <is>
           <t>haemonchus_contortus_prjeb506 (haemonchus contortus)</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr">
+      <c r="I93" t="inlineStr">
         <is>
           <t>GpalpalisIAEA (G. palpalis)</t>
         </is>
@@ -2794,12 +2752,12 @@
           <t>hordeum_vulgare_ft11 (Hordeum vulgare ft11)</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr">
+      <c r="H94" t="inlineStr">
         <is>
           <t>haemonchus_contortus_prjna205202 (haemonchus contortus)</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr">
+      <c r="I94" t="inlineStr">
         <is>
           <t>HasiaticumHyas2018 (H. asiaticum)</t>
         </is>
@@ -2816,12 +2774,12 @@
           <t>hordeum_vulgare_ft144 (Hordeum vulgare ft144)</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr">
+      <c r="H95" t="inlineStr">
         <is>
           <t>haemonchus_placei_prjeb509 (haemonchus placei)</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
+      <c r="I95" t="inlineStr">
         <is>
           <t>Hlongicornis (H. longicornis)</t>
         </is>
@@ -2838,12 +2796,12 @@
           <t>hordeum_vulgare_ft262 (Hordeum vulgare ft262)</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr">
+      <c r="H96" t="inlineStr">
         <is>
           <t>halicephalobus_mephisto_prjna528747 (halicephalobus mephisto)</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr">
+      <c r="I96" t="inlineStr">
         <is>
           <t>HlongicornisHaeL2018 (H. longicornis)</t>
         </is>
@@ -2860,12 +2818,12 @@
           <t>hordeum_vulgare_ft286 (Hordeum vulgare ft286)</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr">
+      <c r="H97" t="inlineStr">
         <is>
           <t>halicephalobus_nkz332_prjna555616 (halicephalobus nkz332)</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
+      <c r="I97" t="inlineStr">
         <is>
           <t>IpersulcatusIper2018 (I. persulcatus)</t>
         </is>
@@ -2882,12 +2840,12 @@
           <t>hordeum_vulgare_ft333 (Hordeum vulgare ft333)</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr">
+      <c r="H98" t="inlineStr">
         <is>
           <t>heligmosomoides_polygyrus_prjeb1203 (heligmosomoides polygyrus)</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
+      <c r="I98" t="inlineStr">
         <is>
           <t>Iricinus (I. ricinus)</t>
         </is>
@@ -2904,12 +2862,12 @@
           <t>hordeum_vulgare_ft628 (Hordeum vulgare ft628)</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr">
+      <c r="H99" t="inlineStr">
         <is>
           <t>heligmosomoides_polygyrus_prjeb15396 (heligmosomoides polygyrus)</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr">
+      <c r="I99" t="inlineStr">
         <is>
           <t>IricinusCharlesRiver (I. ricinus)</t>
         </is>
@@ -2926,12 +2884,12 @@
           <t>hordeum_vulgare_ft67 (Hordeum vulgare ft67)</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr">
+      <c r="H100" t="inlineStr">
         <is>
           <t>heterodera_glycines_prjna381081 (heterodera glycines)</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
+      <c r="I100" t="inlineStr">
         <is>
           <t>Iscapularis (I. scapularis)</t>
         </is>
@@ -2948,12 +2906,12 @@
           <t>hordeum_vulgare_ft880 (Hordeum vulgare ft880)</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr">
+      <c r="H101" t="inlineStr">
         <is>
           <t>heterodera_schachtii_prjna522950 (heterodera schachtii)</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
+      <c r="I101" t="inlineStr">
         <is>
           <t>IscapularisISE6 (I. scapularis)</t>
         </is>
@@ -2970,12 +2928,12 @@
           <t>hordeum_vulgare_goldenmelon (Hordeum vulgare goldenmelon)</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr">
+      <c r="H102" t="inlineStr">
         <is>
           <t>heterodera_schachtii_prjna767548 (heterodera schachtii)</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
+      <c r="I102" t="inlineStr">
         <is>
           <t>IscapularisPalLabHiFi (I. scapularis)</t>
         </is>
@@ -2992,12 +2950,12 @@
           <t>hordeum_vulgare_goldenpromise (Hordeum vulgare goldenpromise)</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr">
+      <c r="H103" t="inlineStr">
         <is>
           <t>heterorhabditis_bacteriophora_prjna13977 (heterorhabditis bacteriophora)</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
+      <c r="I103" t="inlineStr">
         <is>
           <t>IscapularisWikel (I. scapularis)</t>
         </is>
@@ -3014,12 +2972,12 @@
           <t>hordeum_vulgare_hid055 (Hordeum vulgare hid055)</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr">
+      <c r="H104" t="inlineStr">
         <is>
           <t>hydatigera_taeniaeformis_prjeb534 (hydatigera taeniaeformis)</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
+      <c r="I104" t="inlineStr">
         <is>
           <t>Ldeliense (L. deliense)</t>
         </is>
@@ -3036,12 +2994,12 @@
           <t>hordeum_vulgare_hid101 (Hordeum vulgare hid101)</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr">
+      <c r="H105" t="inlineStr">
         <is>
           <t>hymenolepis_diminuta_prjeb30942 (hymenolepis diminuta)</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr">
+      <c r="I105" t="inlineStr">
         <is>
           <t>LdelienseUoL-UT (L. deliense)</t>
         </is>
@@ -3058,12 +3016,12 @@
           <t>hordeum_vulgare_hid249 (Hordeum vulgare hid249)</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr">
+      <c r="H106" t="inlineStr">
         <is>
           <t>hymenolepis_diminuta_prjeb507 (hymenolepis diminuta)</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr">
+      <c r="I106" t="inlineStr">
         <is>
           <t>Llongipalpis (L. longipalpis)</t>
         </is>
@@ -3080,12 +3038,12 @@
           <t>hordeum_vulgare_hid357 (Hordeum vulgare hid357)</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr">
+      <c r="H107" t="inlineStr">
         <is>
           <t>hymenolepis_microstoma_prjeb124 (hymenolepis microstoma)</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr">
+      <c r="I107" t="inlineStr">
         <is>
           <t>LlongipalpisJacobina (L. longipalpis)</t>
         </is>
@@ -3102,12 +3060,12 @@
           <t>hordeum_vulgare_hid380 (Hordeum vulgare hid380)</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="H108" t="inlineStr">
         <is>
           <t>hymenolepis_nana_prjeb508 (hymenolepis nana)</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
+      <c r="I108" t="inlineStr">
         <is>
           <t>LlongipalpisM1 (L. longipalpis)</t>
         </is>
@@ -3124,12 +3082,12 @@
           <t>hordeum_vulgare_hockett (Hordeum vulgare hockett)</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="H109" t="inlineStr">
         <is>
           <t>koerneria_luziae_prjna655932 (koerneria luziae)</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr">
+      <c r="I109" t="inlineStr">
         <is>
           <t>Mdomestica (M. domestica)</t>
         </is>
@@ -3146,12 +3104,12 @@
           <t>hordeum_vulgare_hor10096 (Hordeum vulgare hor10096)</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="H110" t="inlineStr">
         <is>
           <t>levipalatum_texanum_prjna655932 (levipalatum texanum)</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
+      <c r="I110" t="inlineStr">
         <is>
           <t>Mdomesticaaabys (M. domesticaaabys)</t>
         </is>
@@ -3168,12 +3126,12 @@
           <t>hordeum_vulgare_hor10350 (Hordeum vulgare hor10350)</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="H111" t="inlineStr">
         <is>
           <t>linhomoeus_gsco22_prjna953805 (linhomoeus gsco22)</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr">
+      <c r="I111" t="inlineStr">
         <is>
           <t>Mdomesticaaabys2023 (M. domesticaaabys)</t>
         </is>
@@ -3190,12 +3148,12 @@
           <t>hordeum_vulgare_hor10892 (Hordeum vulgare hor10892)</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr">
+      <c r="H112" t="inlineStr">
         <is>
           <t>litomosoides_sigmodontis_prjeb3075 (litomosoides sigmodontis)</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr">
+      <c r="I112" t="inlineStr">
         <is>
           <t>PargentipesIndia (P. argentipes)</t>
         </is>
@@ -3212,12 +3170,12 @@
           <t>hordeum_vulgare_hor1168 (Hordeum vulgare hor1168)</t>
         </is>
       </c>
-      <c r="J113" t="inlineStr">
+      <c r="H113" t="inlineStr">
         <is>
           <t>loa_loa_prjna246086 (loa loa)</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr">
+      <c r="I113" t="inlineStr">
         <is>
           <t>Phumanus (P. humanus)</t>
         </is>
@@ -3234,12 +3192,12 @@
           <t>hordeum_vulgare_hor12184 (Hordeum vulgare hor12184)</t>
         </is>
       </c>
-      <c r="J114" t="inlineStr">
+      <c r="H114" t="inlineStr">
         <is>
           <t>loa_loa_prjna37757 (loa loa)</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
+      <c r="I114" t="inlineStr">
         <is>
           <t>PhumanusUSDA (P. humanus)</t>
         </is>
@@ -3256,12 +3214,12 @@
           <t>hordeum_vulgare_hor12541 (Hordeum vulgare hor12541)</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr">
+      <c r="H115" t="inlineStr">
         <is>
           <t>macrostomum_lignano_prjna284736 (macrostomum lignano)</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr">
+      <c r="I115" t="inlineStr">
         <is>
           <t>Ppapatasi (P. papatasi)</t>
         </is>
@@ -3278,12 +3236,12 @@
           <t>hordeum_vulgare_hor13594 (Hordeum vulgare hor13594)</t>
         </is>
       </c>
-      <c r="J116" t="inlineStr">
+      <c r="H116" t="inlineStr">
         <is>
           <t>macrostomum_lignano_prjna371498 (macrostomum lignano)</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr">
+      <c r="I116" t="inlineStr">
         <is>
           <t>PpapatasiIsrael (P. papatasi)</t>
         </is>
@@ -3300,12 +3258,12 @@
           <t>hordeum_vulgare_hor13663 (Hordeum vulgare hor13663)</t>
         </is>
       </c>
-      <c r="J117" t="inlineStr">
+      <c r="H117" t="inlineStr">
         <is>
           <t>meloidogyne_arenaria_prjeb8714 (meloidogyne arenaria)</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
+      <c r="I117" t="inlineStr">
         <is>
           <t>PpapatasiM1 (P. papatasi)</t>
         </is>
@@ -3322,12 +3280,12 @@
           <t>hordeum_vulgare_hor13821 (Hordeum vulgare hor13821)</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr">
+      <c r="H118" t="inlineStr">
         <is>
           <t>meloidogyne_arenaria_prjna340324 (meloidogyne arenaria)</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr">
+      <c r="I118" t="inlineStr">
         <is>
           <t>Rannulatus (R. annulatus)</t>
         </is>
@@ -3344,12 +3302,12 @@
           <t>hordeum_vulgare_hor13942 (Hordeum vulgare hor13942)</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr">
+      <c r="H119" t="inlineStr">
         <is>
           <t>meloidogyne_arenaria_prjna438575 (meloidogyne arenaria)</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr">
+      <c r="I119" t="inlineStr">
         <is>
           <t>RannulatusKleinGrass (R. annulatus)</t>
         </is>
@@ -3366,12 +3324,12 @@
           <t>hordeum_vulgare_hor14061 (Hordeum vulgare hor14061)</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr">
+      <c r="H120" t="inlineStr">
         <is>
           <t>meloidogyne_enterolobii_prjeb36431 (meloidogyne enterolobii)</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr">
+      <c r="I120" t="inlineStr">
         <is>
           <t>Rmicroplus (R. microplus)</t>
         </is>
@@ -3388,12 +3346,12 @@
           <t>hordeum_vulgare_hor14121 (Hordeum vulgare hor14121)</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr">
+      <c r="H121" t="inlineStr">
         <is>
           <t>meloidogyne_enterolobii_prjna340324 (meloidogyne enterolobii)</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr">
+      <c r="I121" t="inlineStr">
         <is>
           <t>RmicroplusRmic-2018 (R. microplus)</t>
         </is>
@@ -3410,12 +3368,12 @@
           <t>hordeum_vulgare_hor14273 (Hordeum vulgare hor14273)</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr">
+      <c r="H122" t="inlineStr">
         <is>
           <t>meloidogyne_floridensis_prjeb6016 (meloidogyne floridensis)</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr">
+      <c r="I122" t="inlineStr">
         <is>
           <t>Rprolixus (R. prolixus)</t>
         </is>
@@ -3432,12 +3390,12 @@
           <t>hordeum_vulgare_hor1702 (Hordeum vulgare hor1702)</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr">
+      <c r="H123" t="inlineStr">
         <is>
           <t>meloidogyne_floridensis_prjna340324 (meloidogyne floridensis)</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
+      <c r="I123" t="inlineStr">
         <is>
           <t>RprolixusCDC (R. prolixus)</t>
         </is>
@@ -3454,12 +3412,12 @@
           <t>hordeum_vulgare_hor18321 (Hordeum vulgare hor18321)</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr">
+      <c r="H124" t="inlineStr">
         <is>
           <t>meloidogyne_graminicola_prjna411966 (meloidogyne graminicola)</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
+      <c r="I124" t="inlineStr">
         <is>
           <t>RsanguineusRsan-2018 (R. sanguineus)</t>
         </is>
@@ -3476,12 +3434,12 @@
           <t>hordeum_vulgare_hor19184 (Hordeum vulgare hor19184)</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr">
+      <c r="H125" t="inlineStr">
         <is>
           <t>meloidogyne_hapla_prjna29083 (meloidogyne hapla)</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr">
+      <c r="I125" t="inlineStr">
         <is>
           <t>Scalcitrans (S. calcitrans)</t>
         </is>
@@ -3498,12 +3456,12 @@
           <t>hordeum_vulgare_hor21256 (Hordeum vulgare hor21256)</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr">
+      <c r="H126" t="inlineStr">
         <is>
           <t>meloidogyne_incognita_prjeb8714 (meloidogyne incognita)</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr">
+      <c r="I126" t="inlineStr">
         <is>
           <t>ScalcitransUSDA (S. calcitrans)</t>
         </is>
@@ -3520,12 +3478,12 @@
           <t>hordeum_vulgare_hor21322 (Hordeum vulgare hor21322)</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr">
+      <c r="H127" t="inlineStr">
         <is>
           <t>meloidogyne_incognita_prjna340324 (meloidogyne incognita)</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr">
+      <c r="I127" t="inlineStr">
         <is>
           <t>ScyaneusScyaPA1 (S. cyaneus)</t>
         </is>
@@ -3542,12 +3500,12 @@
           <t>hordeum_vulgare_hor21595 (Hordeum vulgare hor21595)</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr">
+      <c r="H128" t="inlineStr">
         <is>
           <t>meloidogyne_javanica_prjeb8714 (meloidogyne javanica)</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr">
+      <c r="I128" t="inlineStr">
         <is>
           <t>Sscabiei (S. scabiei)</t>
         </is>
@@ -3564,12 +3522,12 @@
           <t>hordeum_vulgare_hor21599 (Hordeum vulgare hor21599)</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr">
+      <c r="H129" t="inlineStr">
         <is>
           <t>meloidogyne_javanica_prjna340324 (meloidogyne javanica)</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr">
+      <c r="I129" t="inlineStr">
         <is>
           <t>SscabieiArlian (S. scabiei)</t>
         </is>
@@ -3586,12 +3544,12 @@
           <t>hordeum_vulgare_hor2180 (Hordeum vulgare hor2180)</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr">
+      <c r="H130" t="inlineStr">
         <is>
           <t>mesocestoides_corti_prjeb510 (mesocestoides corti)</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr">
+      <c r="I130" t="inlineStr">
         <is>
           <t>Tinfestans (T. infestans)</t>
         </is>
@@ -3608,12 +3566,12 @@
           <t>hordeum_vulgare_hor2779 (Hordeum vulgare hor2779)</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr">
+      <c r="H131" t="inlineStr">
         <is>
           <t>mesodorylaimus_yzb24_prjna953805 (mesodorylaimus yzb24)</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr">
+      <c r="I131" t="inlineStr">
         <is>
           <t>TinfestansFIOC_28 (T. infestans)</t>
         </is>
@@ -3630,7 +3588,7 @@
           <t>hordeum_vulgare_hor2830 (Hordeum vulgare hor2830)</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr">
+      <c r="H132" t="inlineStr">
         <is>
           <t>mesorhabditis_belari_prjeb61636 (mesorhabditis belari)</t>
         </is>
@@ -3647,7 +3605,7 @@
           <t>hordeum_vulgare_hor3081 (Hordeum vulgare hor3081)</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr">
+      <c r="H133" t="inlineStr">
         <is>
           <t>mesorhabditis_spiculigera_prjeb59059 (mesorhabditis spiculigera)</t>
         </is>
@@ -3664,7 +3622,7 @@
           <t>hordeum_vulgare_hor3365 (Hordeum vulgare hor3365)</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr">
+      <c r="H134" t="inlineStr">
         <is>
           <t>micoletzkya_japonica_prjeb27334 (micoletzkya japonica)</t>
         </is>
@@ -3681,7 +3639,7 @@
           <t>hordeum_vulgare_hor3474 (Hordeum vulgare hor3474)</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr">
+      <c r="H135" t="inlineStr">
         <is>
           <t>microlaimidae_yzb23_prjna953805 (microlaimidae yzb23)</t>
         </is>
@@ -3698,7 +3656,7 @@
           <t>hordeum_vulgare_hor4224 (Hordeum vulgare hor4224)</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr">
+      <c r="H136" t="inlineStr">
         <is>
           <t>necator_americanus_prjna1007425 (necator americanus)</t>
         </is>
@@ -3715,7 +3673,7 @@
           <t>hordeum_vulgare_hor495 (Hordeum vulgare hor495)</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
+      <c r="H137" t="inlineStr">
         <is>
           <t>necator_americanus_prjna72135 (necator americanus)</t>
         </is>
@@ -3732,7 +3690,7 @@
           <t>hordeum_vulgare_hor6220 (Hordeum vulgare hor6220)</t>
         </is>
       </c>
-      <c r="J138" t="inlineStr">
+      <c r="H138" t="inlineStr">
         <is>
           <t>nippostrongylus_brasiliensis_prjeb511 (nippostrongylus brasiliensis)</t>
         </is>
@@ -3749,7 +3707,7 @@
           <t>hordeum_vulgare_hor7172 (Hordeum vulgare hor7172)</t>
         </is>
       </c>
-      <c r="J139" t="inlineStr">
+      <c r="H139" t="inlineStr">
         <is>
           <t>nippostrongylus_brasiliensis_prjna994163 (nippostrongylus brasiliensis)</t>
         </is>
@@ -3766,7 +3724,7 @@
           <t>hordeum_vulgare_hor7385 (Hordeum vulgare hor7385)</t>
         </is>
       </c>
-      <c r="J140" t="inlineStr">
+      <c r="H140" t="inlineStr">
         <is>
           <t>oesophagostomum_dentatum_prjna72579 (oesophagostomum dentatum)</t>
         </is>
@@ -3783,7 +3741,7 @@
           <t>hordeum_vulgare_hor7552 (Hordeum vulgare hor7552)</t>
         </is>
       </c>
-      <c r="J141" t="inlineStr">
+      <c r="H141" t="inlineStr">
         <is>
           <t>onchocerca_flexuosa_prjeb512 (onchocerca flexuosa)</t>
         </is>
@@ -3800,7 +3758,7 @@
           <t>hordeum_vulgare_hor8117 (Hordeum vulgare hor8117)</t>
         </is>
       </c>
-      <c r="J142" t="inlineStr">
+      <c r="H142" t="inlineStr">
         <is>
           <t>onchocerca_flexuosa_prjna230512 (onchocerca flexuosa)</t>
         </is>
@@ -3817,7 +3775,7 @@
           <t>hordeum_vulgare_hor8148 (Hordeum vulgare hor8148)</t>
         </is>
       </c>
-      <c r="J143" t="inlineStr">
+      <c r="H143" t="inlineStr">
         <is>
           <t>onchocerca_ochengi_prjeb1204 (onchocerca ochengi)</t>
         </is>
@@ -3834,7 +3792,7 @@
           <t>hordeum_vulgare_hor9043 (Hordeum vulgare hor9043)</t>
         </is>
       </c>
-      <c r="J144" t="inlineStr">
+      <c r="H144" t="inlineStr">
         <is>
           <t>onchocerca_ochengi_prjeb1465 (onchocerca ochengi)</t>
         </is>
@@ -3851,7 +3809,7 @@
           <t>hordeum_vulgare_hor9972 (Hordeum vulgare hor9972)</t>
         </is>
       </c>
-      <c r="J145" t="inlineStr">
+      <c r="H145" t="inlineStr">
         <is>
           <t>onchocerca_volvulus_prjeb513 (onchocerca volvulus)</t>
         </is>
@@ -3868,7 +3826,7 @@
           <t>hordeum_vulgare_igri (Hordeum vulgare igri)</t>
         </is>
       </c>
-      <c r="J146" t="inlineStr">
+      <c r="H146" t="inlineStr">
         <is>
           <t>opisthorchis_felineus_prjna413383 (opisthorchis felineus)</t>
         </is>
@@ -3885,7 +3843,7 @@
           <t>hordeum_vulgare_maximus (Hordeum vulgare maximus)</t>
         </is>
       </c>
-      <c r="J147" t="inlineStr">
+      <c r="H147" t="inlineStr">
         <is>
           <t>opisthorchis_viverrini_prjna222628 (opisthorchis viverrini)</t>
         </is>
@@ -3902,7 +3860,7 @@
           <t>hordeum_vulgare_oun333 (Hordeum vulgare oun333)</t>
         </is>
       </c>
-      <c r="J148" t="inlineStr">
+      <c r="H148" t="inlineStr">
         <is>
           <t>oscheius_tipulae_prjeb15512 (oscheius tipulae)</t>
         </is>
@@ -3919,7 +3877,7 @@
           <t>hordeum_vulgare_rgtplanet (Hordeum vulgare rgtplanet)</t>
         </is>
       </c>
-      <c r="J149" t="inlineStr">
+      <c r="H149" t="inlineStr">
         <is>
           <t>oscheius_tipulae_prjna644888 (oscheius tipulae)</t>
         </is>
@@ -3936,7 +3894,7 @@
           <t>hordeum_vulgare_tritex (Hordeum vulgare tritex)</t>
         </is>
       </c>
-      <c r="J150" t="inlineStr">
+      <c r="H150" t="inlineStr">
         <is>
           <t>panagrellus_redivivus_prjna186477 (panagrellus redivivus)</t>
         </is>
@@ -3953,7 +3911,7 @@
           <t>hordeum_vulgare_wbdc078 (Hordeum vulgare wbdc078)</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr">
+      <c r="H151" t="inlineStr">
         <is>
           <t>panagrolaimus_davidi_prjeb32708 (panagrolaimus davidi)</t>
         </is>
@@ -3970,7 +3928,7 @@
           <t>hordeum_vulgare_wbdc103 (Hordeum vulgare wbdc103)</t>
         </is>
       </c>
-      <c r="J152" t="inlineStr">
+      <c r="H152" t="inlineStr">
         <is>
           <t>panagrolaimus_es5_prjeb32708 (panagrolaimus es5)</t>
         </is>
@@ -3987,7 +3945,7 @@
           <t>hordeum_vulgare_wbdc133 (Hordeum vulgare wbdc133)</t>
         </is>
       </c>
-      <c r="J153" t="inlineStr">
+      <c r="H153" t="inlineStr">
         <is>
           <t>panagrolaimus_ju765_prjeb32708 (panagrolaimus ju765)</t>
         </is>
@@ -4004,7 +3962,7 @@
           <t>hordeum_vulgare_wbdc184 (Hordeum vulgare wbdc184)</t>
         </is>
       </c>
-      <c r="J154" t="inlineStr">
+      <c r="H154" t="inlineStr">
         <is>
           <t>panagrolaimus_sp1159_prjeb32708 (panagrolaimus sp1159)</t>
         </is>
@@ -4021,7 +3979,7 @@
           <t>hordeum_vulgare_wbdc199 (Hordeum vulgare wbdc199)</t>
         </is>
       </c>
-      <c r="J155" t="inlineStr">
+      <c r="H155" t="inlineStr">
         <is>
           <t>panagrolaimus_superbus_prjeb32708 (panagrolaimus superbus)</t>
         </is>
@@ -4038,7 +3996,7 @@
           <t>hordeum_vulgare_wbdc207 (Hordeum vulgare wbdc207)</t>
         </is>
       </c>
-      <c r="J156" t="inlineStr">
+      <c r="H156" t="inlineStr">
         <is>
           <t>paragonimus_heterotremus_prjna284523 (paragonimus heterotremus)</t>
         </is>
@@ -4055,7 +4013,7 @@
           <t>hordeum_vulgare_wbdc237 (Hordeum vulgare wbdc237)</t>
         </is>
       </c>
-      <c r="J157" t="inlineStr">
+      <c r="H157" t="inlineStr">
         <is>
           <t>paragonimus_kellicotti_prjna179523 (paragonimus kellicotti)</t>
         </is>
@@ -4072,7 +4030,7 @@
           <t>hordeum_vulgare_wbdc348 (Hordeum vulgare wbdc348)</t>
         </is>
       </c>
-      <c r="J158" t="inlineStr">
+      <c r="H158" t="inlineStr">
         <is>
           <t>paragonimus_skrjabinimiyazakii_prjna245325 (paragonimus skrjabinimiyazakii)</t>
         </is>
@@ -4089,7 +4047,7 @@
           <t>hordeum_vulgare_wbdc349 (Hordeum vulgare wbdc349)</t>
         </is>
       </c>
-      <c r="J159" t="inlineStr">
+      <c r="H159" t="inlineStr">
         <is>
           <t>paragonimus_westermani_prjna219632 (paragonimus westermani)</t>
         </is>
@@ -4106,7 +4064,7 @@
           <t>hordeum_vulgare_zdm01467 (Hordeum vulgare zdm01467)</t>
         </is>
       </c>
-      <c r="J160" t="inlineStr">
+      <c r="H160" t="inlineStr">
         <is>
           <t>paragonimus_westermani_prjna454344 (paragonimus westermani)</t>
         </is>
@@ -4123,7 +4081,7 @@
           <t>hordeum_vulgare_zdm02064 (Hordeum vulgare zdm02064)</t>
         </is>
       </c>
-      <c r="J161" t="inlineStr">
+      <c r="H161" t="inlineStr">
         <is>
           <t>paralinhomoeus_gsco26_prjna953805 (paralinhomoeus gsco26)</t>
         </is>
@@ -4140,7 +4098,7 @@
           <t>ipomoea_triloba (Ipomoea triloba)</t>
         </is>
       </c>
-      <c r="J162" t="inlineStr">
+      <c r="H162" t="inlineStr">
         <is>
           <t>parapristionchus_giblindavisi_prjeb53331 (parapristionchus giblindavisi)</t>
         </is>
@@ -4157,7 +4115,7 @@
           <t>juglans_regia (Juglans regia)</t>
         </is>
       </c>
-      <c r="J163" t="inlineStr">
+      <c r="H163" t="inlineStr">
         <is>
           <t>parascaris_equorum_prjeb514 (parascaris equorum)</t>
         </is>
@@ -4174,7 +4132,7 @@
           <t>kalanchoe_fedtschenkoi (Kalanchoe fedtschenkoi)</t>
         </is>
       </c>
-      <c r="J164" t="inlineStr">
+      <c r="H164" t="inlineStr">
         <is>
           <t>parascaris_univalens_prjna386823 (parascaris univalens)</t>
         </is>
@@ -4191,7 +4149,7 @@
           <t>lablab_purpureus_gca030347555v1cm (Lablab purpureus gca030347555v1cm)</t>
         </is>
       </c>
-      <c r="J165" t="inlineStr">
+      <c r="H165" t="inlineStr">
         <is>
           <t>parastrongyloides_trichosuri_prjeb515 (parastrongyloides trichosuri)</t>
         </is>
@@ -4208,7 +4166,7 @@
           <t>lactuca_sativa (Lactuca sativa)</t>
         </is>
       </c>
-      <c r="J166" t="inlineStr">
+      <c r="H166" t="inlineStr">
         <is>
           <t>parelaphostrongylus_tenuis_prjna729714 (parelaphostrongylus tenuis)</t>
         </is>
@@ -4225,7 +4183,7 @@
           <t>lathyrus_sativus (Lathyrus sativus)</t>
         </is>
       </c>
-      <c r="J167" t="inlineStr">
+      <c r="H167" t="inlineStr">
         <is>
           <t>plectus_sambesii_prjna390260 (plectus sambesii)</t>
         </is>
@@ -4242,7 +4200,7 @@
           <t>leersia_perrieri (Leersia perrieri)</t>
         </is>
       </c>
-      <c r="J168" t="inlineStr">
+      <c r="H168" t="inlineStr">
         <is>
           <t>pristionchus_arcanus_prjeb27334 (pristionchus arcanus)</t>
         </is>
@@ -4259,7 +4217,7 @@
           <t>lolium_perenne (Lolium perenne)</t>
         </is>
       </c>
-      <c r="J169" t="inlineStr">
+      <c r="H169" t="inlineStr">
         <is>
           <t>pristionchus_entomophagus_prjeb27334 (pristionchus entomophagus)</t>
         </is>
@@ -4276,7 +4234,7 @@
           <t>lupinus_angustifolius (Lupinus angustifolius)</t>
         </is>
       </c>
-      <c r="J170" t="inlineStr">
+      <c r="H170" t="inlineStr">
         <is>
           <t>pristionchus_exspectatus_prjeb46690 (pristionchus exspectatus)</t>
         </is>
@@ -4293,7 +4251,7 @@
           <t>malus_domestica_golden (Malus domestica golden)</t>
         </is>
       </c>
-      <c r="J171" t="inlineStr">
+      <c r="H171" t="inlineStr">
         <is>
           <t>pristionchus_fissidentatus_prjeb27334 (pristionchus fissidentatus)</t>
         </is>
@@ -4310,7 +4268,7 @@
           <t>manihot_esculenta (Manihot esculenta)</t>
         </is>
       </c>
-      <c r="J172" t="inlineStr">
+      <c r="H172" t="inlineStr">
         <is>
           <t>pristionchus_japonicus_prjeb27334 (pristionchus japonicus)</t>
         </is>
@@ -4327,7 +4285,7 @@
           <t>marchantia_polymorpha (Marchantia polymorpha)</t>
         </is>
       </c>
-      <c r="J173" t="inlineStr">
+      <c r="H173" t="inlineStr">
         <is>
           <t>pristionchus_maxplancki_prjeb27334 (pristionchus maxplancki)</t>
         </is>
@@ -4344,7 +4302,7 @@
           <t>medicago_truncatula (Medicago truncatula)</t>
         </is>
       </c>
-      <c r="J174" t="inlineStr">
+      <c r="H174" t="inlineStr">
         <is>
           <t>pristionchus_mayeri_prjeb27334 (pristionchus mayeri)</t>
         </is>
@@ -4361,7 +4319,7 @@
           <t>musa_acuminata (Musa acuminata)</t>
         </is>
       </c>
-      <c r="J175" t="inlineStr">
+      <c r="H175" t="inlineStr">
         <is>
           <t>pristionchus_pacificus_prjna12644 (pristionchus pacificus)</t>
         </is>
@@ -4378,7 +4336,7 @@
           <t>nicotiana_attenuata (Nicotiana attenuata)</t>
         </is>
       </c>
-      <c r="J176" t="inlineStr">
+      <c r="H176" t="inlineStr">
         <is>
           <t>protopolystoma_xenopodis_prjeb1201 (protopolystoma xenopodis)</t>
         </is>
@@ -4395,7 +4353,7 @@
           <t>nymphaea_colorata (Nymphaea colorata)</t>
         </is>
       </c>
-      <c r="J177" t="inlineStr">
+      <c r="H177" t="inlineStr">
         <is>
           <t>ptycholaimellus_gst110_prjna953805 (ptycholaimellus gst110)</t>
         </is>
@@ -4412,7 +4370,7 @@
           <t>olea_europaea (Olea europaea)</t>
         </is>
       </c>
-      <c r="J178" t="inlineStr">
+      <c r="H178" t="inlineStr">
         <is>
           <t>rhabditophanes_kr3021_prjeb1297 (rhabditophanes kr3021)</t>
         </is>
@@ -4429,7 +4387,7 @@
           <t>olea_europaea_sylvestris (Olea europaea sylvestris)</t>
         </is>
       </c>
-      <c r="J179" t="inlineStr">
+      <c r="H179" t="inlineStr">
         <is>
           <t>rhynchonema_jsb14_prjna953805 (rhynchonema jsb14)</t>
         </is>
@@ -4446,7 +4404,7 @@
           <t>oryza_barthii (Oryza barthii)</t>
         </is>
       </c>
-      <c r="J180" t="inlineStr">
+      <c r="H180" t="inlineStr">
         <is>
           <t>romanomermis_culicivorax_prjeb1358 (romanomermis culicivorax)</t>
         </is>
@@ -4463,7 +4421,7 @@
           <t>oryza_brachyantha (Oryza brachyantha)</t>
         </is>
       </c>
-      <c r="J181" t="inlineStr">
+      <c r="H181" t="inlineStr">
         <is>
           <t>sabatieria_punctata_prjna953805 (sabatieria punctata)</t>
         </is>
@@ -4480,7 +4438,7 @@
           <t>oryza_glaberrima (Oryza glaberrima)</t>
         </is>
       </c>
-      <c r="J182" t="inlineStr">
+      <c r="H182" t="inlineStr">
         <is>
           <t>schistocephalus_solidus_prjeb527 (schistocephalus solidus)</t>
         </is>
@@ -4497,7 +4455,7 @@
           <t>oryza_glumipatula (Oryza glumipatula)</t>
         </is>
       </c>
-      <c r="J183" t="inlineStr">
+      <c r="H183" t="inlineStr">
         <is>
           <t>schistosoma_bovis_prjna451066 (schistosoma bovis)</t>
         </is>
@@ -4514,7 +4472,7 @@
           <t>oryza_indica (Oryza indica)</t>
         </is>
       </c>
-      <c r="J184" t="inlineStr">
+      <c r="H184" t="inlineStr">
         <is>
           <t>schistosoma_curassoni_prjeb44434 (schistosoma curassoni)</t>
         </is>
@@ -4531,7 +4489,7 @@
           <t>oryza_longistaminata (Oryza longistaminata)</t>
         </is>
       </c>
-      <c r="J185" t="inlineStr">
+      <c r="H185" t="inlineStr">
         <is>
           <t>schistosoma_curassoni_prjeb519 (schistosoma curassoni)</t>
         </is>
@@ -4548,7 +4506,7 @@
           <t>oryza_meridionalis (Oryza meridionalis)</t>
         </is>
       </c>
-      <c r="J186" t="inlineStr">
+      <c r="H186" t="inlineStr">
         <is>
           <t>schistosoma_guineensis_prjeb44434 (schistosoma guineensis)</t>
         </is>
@@ -4565,7 +4523,7 @@
           <t>oryza_nivara (Oryza nivara)</t>
         </is>
       </c>
-      <c r="J187" t="inlineStr">
+      <c r="H187" t="inlineStr">
         <is>
           <t>schistosoma_haematobium_prjna78265 (schistosoma haematobium)</t>
         </is>
@@ -4582,7 +4540,7 @@
           <t>oryza_punctata (Oryza punctata)</t>
         </is>
       </c>
-      <c r="J188" t="inlineStr">
+      <c r="H188" t="inlineStr">
         <is>
           <t>schistosoma_japonicum_prjea34885 (schistosoma japonicum)</t>
         </is>
@@ -4599,7 +4557,7 @@
           <t>oryza_rufipogon (Oryza rufipogon)</t>
         </is>
       </c>
-      <c r="J189" t="inlineStr">
+      <c r="H189" t="inlineStr">
         <is>
           <t>schistosoma_japonicum_prjna520774 (schistosoma japonicum)</t>
         </is>
@@ -4616,7 +4574,7 @@
           <t>oryza_sativa (Oryza sativa)</t>
         </is>
       </c>
-      <c r="J190" t="inlineStr">
+      <c r="H190" t="inlineStr">
         <is>
           <t>schistosoma_japonicum_prjna724792 (schistosoma japonicum)</t>
         </is>
@@ -4633,7 +4591,7 @@
           <t>oryza_sativa_arc (Oryza sativa arc)</t>
         </is>
       </c>
-      <c r="J191" t="inlineStr">
+      <c r="H191" t="inlineStr">
         <is>
           <t>schistosoma_mansoni_prjea36577 (schistosoma mansoni)</t>
         </is>
@@ -4650,7 +4608,7 @@
           <t>oryza_sativa_azucena (Oryza sativa azucena)</t>
         </is>
       </c>
-      <c r="J192" t="inlineStr">
+      <c r="H192" t="inlineStr">
         <is>
           <t>schistosoma_margrebowiei_prjeb44434 (schistosoma margrebowiei)</t>
         </is>
@@ -4667,7 +4625,7 @@
           <t>oryza_sativa_chaomeo (Oryza sativa chaomeo)</t>
         </is>
       </c>
-      <c r="J193" t="inlineStr">
+      <c r="H193" t="inlineStr">
         <is>
           <t>schistosoma_mattheei_prjeb44434 (schistosoma mattheei)</t>
         </is>
@@ -4684,7 +4642,7 @@
           <t>oryza_sativa_gobolsailbalam (Oryza sativa gobolsailbalam)</t>
         </is>
       </c>
-      <c r="J194" t="inlineStr">
+      <c r="H194" t="inlineStr">
         <is>
           <t>schistosoma_spindale_prjeb44434 (schistosoma spindale)</t>
         </is>
@@ -4701,7 +4659,7 @@
           <t>oryza_sativa_ir64 (Oryza sativa ir64)</t>
         </is>
       </c>
-      <c r="J195" t="inlineStr">
+      <c r="H195" t="inlineStr">
         <is>
           <t>schistosoma_turkestanicum_prjeb44434 (schistosoma turkestanicum)</t>
         </is>
@@ -4718,7 +4676,7 @@
           <t>oryza_sativa_ketannangka (Oryza sativa ketannangka)</t>
         </is>
       </c>
-      <c r="J196" t="inlineStr">
+      <c r="H196" t="inlineStr">
         <is>
           <t>schmidtea_mediterranea_prjna12585 (schmidtea mediterranea)</t>
         </is>
@@ -4735,7 +4693,7 @@
           <t>oryza_sativa_khaoyaiguang (Oryza sativa khaoyaiguang)</t>
         </is>
       </c>
-      <c r="J197" t="inlineStr">
+      <c r="H197" t="inlineStr">
         <is>
           <t>setaria_digitata_prjna479729 (setaria digitata)</t>
         </is>
@@ -4752,7 +4710,7 @@
           <t>oryza_sativa_larhamugad (Oryza sativa larhamugad)</t>
         </is>
       </c>
-      <c r="J198" t="inlineStr">
+      <c r="H198" t="inlineStr">
         <is>
           <t>soboliphyme_baturini_prjeb516 (soboliphyme baturini)</t>
         </is>
@@ -4769,7 +4727,7 @@
           <t>oryza_sativa_lima (Oryza sativa lima)</t>
         </is>
       </c>
-      <c r="J199" t="inlineStr">
+      <c r="H199" t="inlineStr">
         <is>
           <t>spirometra_erinaceieuropaei_prjeb1202 (spirometra erinaceieuropaei)</t>
         </is>
@@ -4786,7 +4744,7 @@
           <t>oryza_sativa_liuxu (Oryza sativa liuxu)</t>
         </is>
       </c>
-      <c r="J200" t="inlineStr">
+      <c r="H200" t="inlineStr">
         <is>
           <t>steinernema_carpocapsae_prjna202318 (steinernema carpocapsae)</t>
         </is>
@@ -4803,7 +4761,7 @@
           <t>oryza_sativa_mh63 (Oryza sativa mh63)</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr">
+      <c r="H201" t="inlineStr">
         <is>
           <t>steinernema_feltiae_prjna204661 (steinernema feltiae)</t>
         </is>
@@ -4820,7 +4778,7 @@
           <t>oryza_sativa_n22 (Oryza sativa n22)</t>
         </is>
       </c>
-      <c r="J202" t="inlineStr">
+      <c r="H202" t="inlineStr">
         <is>
           <t>steinernema_feltiae_prjna353610 (steinernema feltiae)</t>
         </is>
@@ -4837,7 +4795,7 @@
           <t>oryza_sativa_natelboro (Oryza sativa natelboro)</t>
         </is>
       </c>
-      <c r="J203" t="inlineStr">
+      <c r="H203" t="inlineStr">
         <is>
           <t>steinernema_glaseri_prjna204943 (steinernema glaseri)</t>
         </is>
@@ -4854,7 +4812,7 @@
           <t>oryza_sativa_pr106 (Oryza sativa pr106)</t>
         </is>
       </c>
-      <c r="J204" t="inlineStr">
+      <c r="H204" t="inlineStr">
         <is>
           <t>steinernema_hermaphroditum_prjna982879 (steinernema hermaphroditum)</t>
         </is>
@@ -4871,7 +4829,7 @@
           <t>oryza_sativa_zs97 (Oryza sativa zs97)</t>
         </is>
       </c>
-      <c r="J205" t="inlineStr">
+      <c r="H205" t="inlineStr">
         <is>
           <t>steinernema_monticolum_prjna205067 (steinernema monticolum)</t>
         </is>
@@ -4888,7 +4846,7 @@
           <t>ostreococcus_lucimarinus (Ostreococcus lucimarinus)</t>
         </is>
       </c>
-      <c r="J206" t="inlineStr">
+      <c r="H206" t="inlineStr">
         <is>
           <t>steinernema_scapterisci_prjna204942 (steinernema scapterisci)</t>
         </is>
@@ -4905,7 +4863,7 @@
           <t>panicum_hallii (Panicum hallii)</t>
         </is>
       </c>
-      <c r="J207" t="inlineStr">
+      <c r="H207" t="inlineStr">
         <is>
           <t>strongyloides_papillosus_prjeb525 (strongyloides papillosus)</t>
         </is>
@@ -4922,7 +4880,7 @@
           <t>panicum_hallii_fil2 (Panicum hallii fil2)</t>
         </is>
       </c>
-      <c r="J208" t="inlineStr">
+      <c r="H208" t="inlineStr">
         <is>
           <t>strongyloides_ratti_prjeb125 (strongyloides ratti)</t>
         </is>
@@ -4939,7 +4897,7 @@
           <t>papaver_somniferum (Papaver somniferum)</t>
         </is>
       </c>
-      <c r="J209" t="inlineStr">
+      <c r="H209" t="inlineStr">
         <is>
           <t>strongyloides_stercoralis_prjeb528 (strongyloides stercoralis)</t>
         </is>
@@ -4956,7 +4914,7 @@
           <t>phaseolus_vulgaris (Phaseolus vulgaris)</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr">
+      <c r="H210" t="inlineStr">
         <is>
           <t>strongyloides_stercoralis_prjna930454 (strongyloides stercoralis)</t>
         </is>
@@ -4973,7 +4931,7 @@
           <t>physcomitrium_patens (Physcomitrium patens)</t>
         </is>
       </c>
-      <c r="J211" t="inlineStr">
+      <c r="H211" t="inlineStr">
         <is>
           <t>strongyloides_venezuelensis_prjeb530 (strongyloides venezuelensis)</t>
         </is>
@@ -4990,7 +4948,7 @@
           <t>pistacia_vera (Pistacia vera)</t>
         </is>
       </c>
-      <c r="J212" t="inlineStr">
+      <c r="H212" t="inlineStr">
         <is>
           <t>strongylus_vulgaris_prjeb531 (strongylus vulgaris)</t>
         </is>
@@ -5007,7 +4965,7 @@
           <t>pisum_sativum (Pisum sativum)</t>
         </is>
       </c>
-      <c r="J213" t="inlineStr">
+      <c r="H213" t="inlineStr">
         <is>
           <t>syphacia_muris_prjeb524 (syphacia muris)</t>
         </is>
@@ -5024,7 +4982,7 @@
           <t>pisum_sativum_gca024323335v2gb (Pisum sativum gca024323335v2gb)</t>
         </is>
       </c>
-      <c r="J214" t="inlineStr">
+      <c r="H214" t="inlineStr">
         <is>
           <t>taenia_asiatica_prjeb532 (taenia asiatica)</t>
         </is>
@@ -5041,7 +4999,7 @@
           <t>pisum_sativum_gca964186695v1gb (Pisum sativum gca964186695v1gb)</t>
         </is>
       </c>
-      <c r="J215" t="inlineStr">
+      <c r="H215" t="inlineStr">
         <is>
           <t>taenia_asiatica_prjna299871 (taenia asiatica)</t>
         </is>
@@ -5058,7 +5016,7 @@
           <t>populus_trichocarpa (Populus trichocarpa)</t>
         </is>
       </c>
-      <c r="J216" t="inlineStr">
+      <c r="H216" t="inlineStr">
         <is>
           <t>taenia_multiceps_prjna307624 (taenia multiceps)</t>
         </is>
@@ -5075,7 +5033,7 @@
           <t>prunus_avium (Prunus avium)</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr">
+      <c r="H217" t="inlineStr">
         <is>
           <t>taenia_saginata_prjna71493 (taenia saginata)</t>
         </is>
@@ -5092,7 +5050,7 @@
           <t>prunus_dulcis (Prunus dulcis)</t>
         </is>
       </c>
-      <c r="J218" t="inlineStr">
+      <c r="H218" t="inlineStr">
         <is>
           <t>taenia_solium_prjna170813 (taenia solium)</t>
         </is>
@@ -5109,7 +5067,7 @@
           <t>prunus_persica (Prunus persica)</t>
         </is>
       </c>
-      <c r="J219" t="inlineStr">
+      <c r="H219" t="inlineStr">
         <is>
           <t>teladorsagia_circumcincta_prjna72569 (teladorsagia circumcincta)</t>
         </is>
@@ -5126,7 +5084,7 @@
           <t>quercus_lobata (Quercus lobata)</t>
         </is>
       </c>
-      <c r="J220" t="inlineStr">
+      <c r="H220" t="inlineStr">
         <is>
           <t>thelazia_callipaeda_prjeb1205 (thelazia callipaeda)</t>
         </is>
@@ -5143,7 +5101,7 @@
           <t>quercus_suber (Quercus suber)</t>
         </is>
       </c>
-      <c r="J221" t="inlineStr">
+      <c r="H221" t="inlineStr">
         <is>
           <t>theristus_lff411_prjna953805 (theristus lff411)</t>
         </is>
@@ -5160,7 +5118,7 @@
           <t>rosa_chinensis (Rosa chinensis)</t>
         </is>
       </c>
-      <c r="J222" t="inlineStr">
+      <c r="H222" t="inlineStr">
         <is>
           <t>toxocara_canis_prjeb533 (toxocara canis)</t>
         </is>
@@ -5177,7 +5135,7 @@
           <t>saccharum_spontaneum (Saccharum spontaneum)</t>
         </is>
       </c>
-      <c r="J223" t="inlineStr">
+      <c r="H223" t="inlineStr">
         <is>
           <t>toxocara_canis_prjna248777 (toxocara canis)</t>
         </is>
@@ -5194,7 +5152,7 @@
           <t>secale_cereale (Secale cereale)</t>
         </is>
       </c>
-      <c r="J224" t="inlineStr">
+      <c r="H224" t="inlineStr">
         <is>
           <t>trichinella_britovi_prjna257433 (trichinella britovi)</t>
         </is>
@@ -5211,7 +5169,7 @@
           <t>selaginella_moellendorffii (Selaginella moellendorffii)</t>
         </is>
       </c>
-      <c r="J225" t="inlineStr">
+      <c r="H225" t="inlineStr">
         <is>
           <t>trichinella_murrelli_prjna257433 (trichinella murrelli)</t>
         </is>
@@ -5228,7 +5186,7 @@
           <t>sesamum_indicum (Sesamum indicum)</t>
         </is>
       </c>
-      <c r="J226" t="inlineStr">
+      <c r="H226" t="inlineStr">
         <is>
           <t>trichinella_nativa_prjna179527 (trichinella nativa)</t>
         </is>
@@ -5245,7 +5203,7 @@
           <t>setaria_italica (Setaria italica)</t>
         </is>
       </c>
-      <c r="J227" t="inlineStr">
+      <c r="H227" t="inlineStr">
         <is>
           <t>trichinella_nativa_prjna257433 (trichinella nativa)</t>
         </is>
@@ -5262,7 +5220,7 @@
           <t>setaria_viridis (Setaria viridis)</t>
         </is>
       </c>
-      <c r="J228" t="inlineStr">
+      <c r="H228" t="inlineStr">
         <is>
           <t>trichinella_nelsoni_prjna257433 (trichinella nelsoni)</t>
         </is>
@@ -5279,7 +5237,7 @@
           <t>solanum_lycopersicum (Solanum lycopersicum)</t>
         </is>
       </c>
-      <c r="J229" t="inlineStr">
+      <c r="H229" t="inlineStr">
         <is>
           <t>trichinella_papuae_prjna257433 (trichinella papuae)</t>
         </is>
@@ -5296,7 +5254,7 @@
           <t>solanum_tuberosum (Solanum tuberosum)</t>
         </is>
       </c>
-      <c r="J230" t="inlineStr">
+      <c r="H230" t="inlineStr">
         <is>
           <t>trichinella_patagoniensis_prjna257433 (trichinella patagoniensis)</t>
         </is>
@@ -5313,7 +5271,7 @@
           <t>solanum_tuberosum_rh8903916 (Solanum tuberosum rh8903916)</t>
         </is>
       </c>
-      <c r="J231" t="inlineStr">
+      <c r="H231" t="inlineStr">
         <is>
           <t>trichinella_spiralis_prjna12603 (trichinella spiralis)</t>
         </is>
@@ -5330,7 +5288,7 @@
           <t>sorghum_bicolor (Sorghum bicolor)</t>
         </is>
       </c>
-      <c r="J232" t="inlineStr">
+      <c r="H232" t="inlineStr">
         <is>
           <t>trichinella_spiralis_prjna257433 (trichinella spiralis)</t>
         </is>
@@ -5347,7 +5305,7 @@
           <t>sphenostylis_stenocarpa (Sphenostylis stenocarpa)</t>
         </is>
       </c>
-      <c r="J233" t="inlineStr">
+      <c r="H233" t="inlineStr">
         <is>
           <t>trichinella_t6_prjna257433 (trichinella t6)</t>
         </is>
@@ -5364,7 +5322,7 @@
           <t>theobroma_cacao (Theobroma cacao)</t>
         </is>
       </c>
-      <c r="J234" t="inlineStr">
+      <c r="H234" t="inlineStr">
         <is>
           <t>trichinella_t8_prjna257433 (trichinella t8)</t>
         </is>
@@ -5381,7 +5339,7 @@
           <t>theobroma_cacao_criollo (Theobroma cacao criollo)</t>
         </is>
       </c>
-      <c r="J235" t="inlineStr">
+      <c r="H235" t="inlineStr">
         <is>
           <t>trichinella_t9_prjna257433 (trichinella t9)</t>
         </is>
@@ -5398,7 +5356,7 @@
           <t>trifolium_pratense (Trifolium pratense)</t>
         </is>
       </c>
-      <c r="J236" t="inlineStr">
+      <c r="H236" t="inlineStr">
         <is>
           <t>trichinella_zimbabwensis_prjna257433 (trichinella zimbabwensis)</t>
         </is>
@@ -5415,7 +5373,7 @@
           <t>triticum_aestivum (Triticum aestivum)</t>
         </is>
       </c>
-      <c r="J237" t="inlineStr">
+      <c r="H237" t="inlineStr">
         <is>
           <t>trichobilharzia_regenti_prjeb44434 (trichobilharzia regenti)</t>
         </is>
@@ -5432,7 +5390,7 @@
           <t>triticum_aestivum_alchemy (Triticum aestivum alchemy)</t>
         </is>
       </c>
-      <c r="J238" t="inlineStr">
+      <c r="H238" t="inlineStr">
         <is>
           <t>trichobilharzia_szidati_prjeb44434 (trichobilharzia szidati)</t>
         </is>
@@ -5449,7 +5407,7 @@
           <t>triticum_aestivum_arinalrfor (Triticum aestivum arinalrfor)</t>
         </is>
       </c>
-      <c r="J239" t="inlineStr">
+      <c r="H239" t="inlineStr">
         <is>
           <t>trichuris_muris_prjeb126 (trichuris muris)</t>
         </is>
@@ -5466,7 +5424,7 @@
           <t>triticum_aestivum_cadenza (Triticum aestivum cadenza)</t>
         </is>
       </c>
-      <c r="J240" t="inlineStr">
+      <c r="H240" t="inlineStr">
         <is>
           <t>trichuris_suis_prjna179528 (trichuris suis)</t>
         </is>
@@ -5483,7 +5441,7 @@
           <t>triticum_aestivum_claire (Triticum aestivum claire)</t>
         </is>
       </c>
-      <c r="J241" t="inlineStr">
+      <c r="H241" t="inlineStr">
         <is>
           <t>trichuris_suis_prjna208415 (trichuris suis)</t>
         </is>
@@ -5500,7 +5458,7 @@
           <t>triticum_aestivum_jagger (Triticum aestivum jagger)</t>
         </is>
       </c>
-      <c r="J242" t="inlineStr">
+      <c r="H242" t="inlineStr">
         <is>
           <t>trichuris_suis_prjna208416 (trichuris suis)</t>
         </is>
@@ -5517,7 +5475,7 @@
           <t>triticum_aestivum_julius (Triticum aestivum julius)</t>
         </is>
       </c>
-      <c r="J243" t="inlineStr">
+      <c r="H243" t="inlineStr">
         <is>
           <t>trichuris_trichiura_prjeb535 (trichuris trichiura)</t>
         </is>
@@ -5534,7 +5492,7 @@
           <t>triticum_aestivum_kariega (Triticum aestivum kariega)</t>
         </is>
       </c>
-      <c r="J244" t="inlineStr">
+      <c r="H244" t="inlineStr">
         <is>
           <t>trileptium_ribeirensis_prjna953805 (trileptium ribeirensis)</t>
         </is>
@@ -5551,7 +5509,7 @@
           <t>triticum_aestivum_lancer (Triticum aestivum lancer)</t>
         </is>
       </c>
-      <c r="J245" t="inlineStr">
+      <c r="H245" t="inlineStr">
         <is>
           <t>trissonchulus_latispiculum_prjna953805 (trissonchulus latispiculum)</t>
         </is>
@@ -5568,7 +5526,7 @@
           <t>triticum_aestivum_landmark (Triticum aestivum landmark)</t>
         </is>
       </c>
-      <c r="J246" t="inlineStr">
+      <c r="H246" t="inlineStr">
         <is>
           <t>trissonchulus_wlg14_prjna953805 (trissonchulus wlg14)</t>
         </is>
@@ -5585,7 +5543,7 @@
           <t>triticum_aestivum_mace (Triticum aestivum mace)</t>
         </is>
       </c>
-      <c r="J247" t="inlineStr">
+      <c r="H247" t="inlineStr">
         <is>
           <t>wuchereria_bancrofti_prjeb536 (wuchereria bancrofti)</t>
         </is>
@@ -5602,7 +5560,7 @@
           <t>triticum_aestivum_mattis (Triticum aestivum mattis)</t>
         </is>
       </c>
-      <c r="J248" t="inlineStr">
+      <c r="H248" t="inlineStr">
         <is>
           <t>wuchereria_bancrofti_prjna275548 (wuchereria bancrofti)</t>
         </is>

</xml_diff>

<commit_message>
Add manifest note that valid IDs beyond dropdown are supported
</commit_message>
<xml_diff>
--- a/workspace/input/input_generation/download_plan.xlsx
+++ b/workspace/input/input_generation/download_plan.xlsx
@@ -137,6 +137,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>genegalleon</author>
+  </authors>
+  <commentList>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>IDs not listed in the drop-down are still supported if they are valid in the provider database.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -518,6 +533,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Expand CNGB dropdown examples to five IDs
</commit_message>
<xml_diff>
--- a/workspace/input/input_generation/download_plan.xlsx
+++ b/workspace/input/input_generation/download_plan.xlsx
@@ -15,7 +15,7 @@
     <definedName name="id_opts_ensemblplants">'_lists'!$C$1:$C$266</definedName>
     <definedName name="id_opts_ncbi">'_lists'!$D$1:$D$5</definedName>
     <definedName name="id_opts_coge">'_lists'!$E$1:$E$5</definedName>
-    <definedName name="id_opts_cngb">'_lists'!$F$1:$F$1</definedName>
+    <definedName name="id_opts_cngb">'_lists'!$F$1:$F$5</definedName>
     <definedName name="id_opts_flybase">'_lists'!$G$1:$G$12</definedName>
     <definedName name="id_opts_wormbase">'_lists'!$H$1:$H$248</definedName>
     <definedName name="id_opts_vectorbase">'_lists'!$I$1:$I$131</definedName>
@@ -624,6 +624,11 @@
           <t>29177 (Oryza sativa)</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>GCF_000001405.40 (Homo sapiens)</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>dere_r1.05 (Drosophila erecta)</t>
@@ -666,6 +671,11 @@
           <t>42091 (Zea mays)</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>GCA_000001635.9 (Mus musculus)</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>dgri_r1.05 (Drosophila grimshawi)</t>
@@ -708,6 +718,11 @@
           <t>78085 (Drosophila melanogaster)</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>GCF_049306965.1 (Danio rerio)</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>dmel_r6.66 (Drosophila melanogaster)</t>
@@ -748,6 +763,11 @@
       <c r="E5" t="inlineStr">
         <is>
           <t>72417 (Caenorhabditis elegans)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GCA_000001215.4 (Drosophila melanogaster)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">

</xml_diff>

<commit_message>
Improve workflow templates and enum modes
</commit_message>
<xml_diff>
--- a/workspace/input/input_generation/download_plan.xlsx
+++ b/workspace/input/input_generation/download_plan.xlsx
@@ -19,7 +19,8 @@
     <definedName name="id_opts_flybase">'_lists'!$G$1:$G$12</definedName>
     <definedName name="id_opts_wormbase">'_lists'!$H$1:$H$248</definedName>
     <definedName name="id_opts_vectorbase">'_lists'!$I$1:$I$131</definedName>
-    <definedName name="id_opts_local">'_lists'!$J$1:$J$1</definedName>
+    <definedName name="id_opts_fernbase">'_lists'!$J$1:$J$2</definedName>
+    <definedName name="id_opts_local">'_lists'!$K$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -145,9 +146,135 @@
     <author>genegalleon</author>
   </authors>
   <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>Required.
+Allowed values: ensembl, ensemblplants, ncbi, coge, cngb, flybase, wormbase, vectorbase, fernbase, local.
+Use the drop-down when possible.
+In XLSX templates this must remain the first column.</t>
+      </text>
+    </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>IDs not listed in the drop-down are still supported if they are valid in the provider database.</t>
+        <t>Required.
+Provider-specific identifier.
+Examples:
+- ensembl: homo_sapiens
+- ncbi: GCF_000001405.40 or GCA_000001635.9
+- coge: numeric genome_id (gid), for example 24739
+- cngb: CNA... or GCA/GCF accession
+- local: local species directory ID or path-style ID
+The drop-down is provider-specific, but any valid value can still be typed manually.
+For non-local providers, labels like 'GCF_000001405.40 (Homo sapiens)' are accepted;
+the parser uses the token before the first space as the actual ID.
+In XLSX templates this must remain the second column.</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Stable species label used for output directories and filename templating.
+Recommended format: letters, numbers, and underscores only, for example Homo_sapiens.
+If blank, it is inferred from provider metadata, local directory names, or id when possible.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>Conditionally required.
+URL to the CDS FASTA file.
+Accepted schemes: https://, http://, ftp://, file://.
+Leave blank when provider/id auto-resolution or cds_url_template will fill it.
+Typical suffixes: .fa, .fasta, .fna with optional .gz.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Conditionally required.
+URL to the annotation file.
+Accepted schemes: https://, http://, ftp://, file://.
+Leave blank when provider/id auto-resolution or gff_url_template will fill it.
+Typical suffixes: .gff, .gff3, .gtf with optional .gz.</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional but recommended for genome-aware workflows.
+URL to the genome FASTA file.
+Accepted schemes: https://, http://, ftp://, file://.
+Leave blank to skip genome download; provider/id auto-resolution or genome_url_template can fill it.
+Typical suffixes: .fa, .fasta, .fna with optional .gz.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Output filename used when the CDS file is written to the raw download directory.
+Use a basename only, not a directory path.
+If blank, it is inferred from cds_url or provider metadata.</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Output filename used when the GFF/GTF file is written to the raw download directory.
+Use a basename only, not a directory path.
+If blank, it is inferred from gff_url or provider metadata.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Output filename used when the genome FASTA is written to the raw download directory.
+Use a basename only, not a directory path.
+If blank, it is inferred from genome_url or provider metadata.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Template used to build cds_url when cds_url is blank.
+Supported placeholders: {id}, {species_key}, {provider}.
+Example: https://example.org/{species_key}/{id}.cds.fa.gz</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Template used to build gff_url when gff_url is blank.
+Supported placeholders: {id}, {species_key}, {provider}.
+Example: https://example.org/{species_key}/{id}.gff3.gz</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional.
+Template used to build genome_url when genome_url is blank.
+Supported placeholders: {id}, {species_key}, {provider}.
+Example: https://example.org/{species_key}/{id}.genome.fa.gz</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional; mainly for provider=local.
+Absolute path or path relative to this manifest file.
+Converted to file:// at runtime.
+Use this when the CDS already exists locally and you do not want to write cds_url manually.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional; mainly for provider=local.
+Absolute path or path relative to this manifest file.
+Converted to file:// at runtime.
+Use this when the annotation file already exists locally and you do not want to write gff_url manually.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional; mainly for provider=local.
+Absolute path or path relative to this manifest file.
+Converted to file:// at runtime.
+Use this when the genome FASTA already exists locally and you do not want to write genome_url manually.</t>
       </text>
     </comment>
   </commentList>
@@ -526,7 +653,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="A2:A5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>=_lists!$A$1:$A$9</formula1>
+      <formula1>=_lists!$A$1:$A$10</formula1>
     </dataValidation>
     <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="ID candidates" error="This drop-down changes by provider. For provider=ncbi, five model-organism IDs are shown as examples. You can still type any other ID value." type="list" errorStyle="information">
       <formula1>=INDIRECT("id_opts_"&amp;$A2)</formula1>
@@ -543,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J348"/>
+  <dimension ref="A1:K348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,6 +721,11 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>Azolla_filiculoides (Azolla filiculoides)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>/absolute/path/to/local/species_dir</t>
         </is>
       </c>
@@ -644,6 +776,11 @@
           <t>AaegyptiAag2 (A. aegypti)</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Salvinia_cucullata_v2 (Salvinia cucullata v2)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -885,36 +1022,41 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>fernbase</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>anas_platyrhynchos (Mallard)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>arabis_alpina (Arabis alpina)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>dsim_r2.02 (Drosophila simulans)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>angiostrongylus_cantonensis_prjna350391 (angiostrongylus cantonensis)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>AalbopictusFoshan (A. albopictus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>local</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>anas_platyrhynchos (Mallard)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>arabis_alpina (Arabis alpina)</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>dsim_r2.02 (Drosophila simulans)</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>angiostrongylus_cantonensis_prjna350391 (angiostrongylus cantonensis)</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>AalbopictusFoshan (A. albopictus)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
       <c r="B10" t="inlineStr">
         <is>
           <t>anas_platyrhynchos_platyrhynchos (Duck)</t>

</xml_diff>